<commit_message>
Updated excel format output with airline crew
</commit_message>
<xml_diff>
--- a/ScheduleTemplate.xlsx
+++ b/ScheduleTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brian/Documents/Projects/Work Scheduler V2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E50885F0-4E5E-A44C-AE04-9B6C70D6F2E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9352C86-615A-0C46-8BC3-AE5FDB0E3AD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="860" windowWidth="25620" windowHeight="21380" xr2:uid="{880B7373-6B33-44EB-8E47-BB6DFBBF0420}"/>
+    <workbookView xWindow="8560" yWindow="800" windowWidth="25640" windowHeight="21420" xr2:uid="{880B7373-6B33-44EB-8E47-BB6DFBBF0420}"/>
   </bookViews>
   <sheets>
     <sheet name="June 19 - June 25" sheetId="1" r:id="rId1"/>
@@ -35,14 +35,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="60">
   <si>
     <t>Holiday Inn Express Vancouver Airport - Schedule</t>
   </si>
   <si>
-    <t>* = Frist Aid Cert</t>
-  </si>
-  <si>
     <t>THU</t>
   </si>
   <si>
@@ -178,37 +175,46 @@
     <t>Back Up</t>
   </si>
   <si>
-    <t>TERRY</t>
-  </si>
-  <si>
-    <t>TRISTAN</t>
-  </si>
-  <si>
     <t>SATO</t>
   </si>
   <si>
-    <t>TBD</t>
-  </si>
-  <si>
-    <t>VICTOR</t>
-  </si>
-  <si>
-    <t>TONY H</t>
-  </si>
-  <si>
     <t>TOSHIYUKI</t>
   </si>
   <si>
-    <t>WILLEM</t>
-  </si>
-  <si>
-    <t>IGOR</t>
-  </si>
-  <si>
     <t>ANNA</t>
   </si>
   <si>
     <t>JOJO</t>
+  </si>
+  <si>
+    <t>RAPHAEL</t>
+  </si>
+  <si>
+    <t>TERRY*</t>
+  </si>
+  <si>
+    <t>TRISTAN*</t>
+  </si>
+  <si>
+    <t>**OCC</t>
+  </si>
+  <si>
+    <t>* = First Aid Cert</t>
+  </si>
+  <si>
+    <t>** SUB TO CHANGE</t>
+  </si>
+  <si>
+    <t>ROBENSON*</t>
+  </si>
+  <si>
+    <t>MING</t>
+  </si>
+  <si>
+    <t>**AEROMEX</t>
+  </si>
+  <si>
+    <t>**SKYWEST</t>
   </si>
 </sst>
 </file>
@@ -369,7 +375,7 @@
       <name val="Bahnschrift SemiBold"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -379,6 +385,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -542,7 +566,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -640,21 +664,6 @@
     <xf numFmtId="9" fontId="19" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="19" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -673,27 +682,30 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="16" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -718,19 +730,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -764,9 +770,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1107,7 +1110,7 @@
     <tabColor theme="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:R75"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="9.1640625" style="4"/>
@@ -1129,16 +1132,16 @@
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="52" t="s">
+      <c r="D1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-      <c r="I1" s="52"/>
-      <c r="J1" s="52"/>
-      <c r="K1" s="52"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
       <c r="L1" s="2"/>
       <c r="M1" s="3"/>
       <c r="N1" s="3"/>
@@ -1166,7 +1169,7 @@
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="6" t="s">
-        <v>1</v>
+        <v>54</v>
       </c>
       <c r="E3" s="7">
         <v>45827</v>
@@ -1189,7 +1192,7 @@
       <c r="K3" s="7">
         <v>45833</v>
       </c>
-      <c r="L3" s="40"/>
+      <c r="L3" s="35"/>
       <c r="M3" s="8"/>
       <c r="N3" s="8"/>
       <c r="O3" s="8"/>
@@ -1201,27 +1204,29 @@
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
-      <c r="D4" s="9"/>
+      <c r="D4" s="9" t="s">
+        <v>55</v>
+      </c>
       <c r="E4" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="G4" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="H4" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="I4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="J4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="K4" s="10" t="s">
         <v>7</v>
-      </c>
-      <c r="K4" s="10" t="s">
-        <v>8</v>
       </c>
       <c r="L4" s="6"/>
       <c r="M4" s="11"/>
@@ -1232,13 +1237,13 @@
       <c r="R4" s="11"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A5" s="53" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="54"/>
-      <c r="C5" s="55"/>
+      <c r="A5" s="49" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="50"/>
+      <c r="C5" s="51"/>
       <c r="D5" s="13" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" s="14"/>
       <c r="F5" s="14"/>
@@ -1247,7 +1252,7 @@
       <c r="I5" s="14"/>
       <c r="J5" s="14"/>
       <c r="K5" s="14"/>
-      <c r="L5" s="41"/>
+      <c r="L5" s="36"/>
       <c r="M5" s="11"/>
       <c r="N5" s="12"/>
       <c r="O5" s="11"/>
@@ -1256,9 +1261,9 @@
       <c r="R5" s="11"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A6" s="56"/>
-      <c r="B6" s="57"/>
-      <c r="C6" s="58"/>
+      <c r="A6" s="52"/>
+      <c r="B6" s="53"/>
+      <c r="C6" s="54"/>
       <c r="D6" s="13" t="s">
         <v>12</v>
       </c>
@@ -1269,7 +1274,7 @@
       <c r="I6" s="14"/>
       <c r="J6" s="14"/>
       <c r="K6" s="25"/>
-      <c r="L6" s="41"/>
+      <c r="L6" s="36"/>
       <c r="M6" s="11"/>
       <c r="N6" s="12"/>
       <c r="O6" s="11"/>
@@ -1278,11 +1283,11 @@
       <c r="R6" s="11"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A7" s="56"/>
-      <c r="B7" s="57"/>
-      <c r="C7" s="58"/>
+      <c r="A7" s="52"/>
+      <c r="B7" s="53"/>
+      <c r="C7" s="54"/>
       <c r="D7" s="13" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
       <c r="E7" s="14"/>
       <c r="F7" s="14"/>
@@ -1291,7 +1296,7 @@
       <c r="I7" s="14"/>
       <c r="J7" s="25"/>
       <c r="K7" s="14"/>
-      <c r="L7" s="41"/>
+      <c r="L7" s="36"/>
       <c r="M7" s="11"/>
       <c r="N7" s="12"/>
       <c r="O7" s="11"/>
@@ -1300,63 +1305,59 @@
       <c r="R7" s="11"/>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A8" s="56"/>
-      <c r="B8" s="57"/>
-      <c r="C8" s="58"/>
-      <c r="D8" s="13" t="s">
-        <v>15</v>
-      </c>
+      <c r="A8" s="52"/>
+      <c r="B8" s="53"/>
+      <c r="C8" s="54"/>
+      <c r="D8" s="13"/>
       <c r="E8" s="14"/>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
       <c r="H8" s="14"/>
       <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
+      <c r="J8" s="25"/>
       <c r="K8" s="14"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="15"/>
+      <c r="L8" s="36"/>
+      <c r="M8" s="11"/>
       <c r="N8" s="12"/>
-      <c r="O8" s="16"/>
-      <c r="P8" s="16"/>
-      <c r="Q8" s="16"/>
-      <c r="R8" s="16"/>
-    </row>
-    <row r="9" spans="1:18" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="56"/>
-      <c r="B9" s="57"/>
-      <c r="C9" s="58"/>
-      <c r="D9" s="59" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9" s="60"/>
-      <c r="F9" s="60"/>
-      <c r="G9" s="60"/>
-      <c r="H9" s="60"/>
-      <c r="I9" s="60"/>
-      <c r="J9" s="60"/>
-      <c r="K9" s="61"/>
+      <c r="O8" s="11"/>
+      <c r="P8" s="11"/>
+      <c r="Q8" s="11"/>
+      <c r="R8" s="11"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A9" s="52"/>
+      <c r="B9" s="53"/>
+      <c r="C9" s="54"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
       <c r="L9" s="6"/>
       <c r="M9" s="15"/>
       <c r="N9" s="12"/>
-      <c r="O9" s="15"/>
-      <c r="P9" s="15"/>
-      <c r="Q9" s="15"/>
-      <c r="R9" s="15"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A10" s="56"/>
-      <c r="B10" s="57"/>
-      <c r="C10" s="58"/>
-      <c r="D10" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
-      <c r="K10" s="14"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="16"/>
+      <c r="Q9" s="16"/>
+      <c r="R9" s="16"/>
+    </row>
+    <row r="10" spans="1:18" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="52"/>
+      <c r="B10" s="53"/>
+      <c r="C10" s="54"/>
+      <c r="D10" s="55" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="56"/>
+      <c r="F10" s="56"/>
+      <c r="G10" s="56"/>
+      <c r="H10" s="56"/>
+      <c r="I10" s="56"/>
+      <c r="J10" s="56"/>
+      <c r="K10" s="57"/>
       <c r="L10" s="6"/>
       <c r="M10" s="15"/>
       <c r="N10" s="12"/>
@@ -1366,11 +1367,11 @@
       <c r="R10" s="15"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A11" s="56"/>
-      <c r="B11" s="57"/>
-      <c r="C11" s="58"/>
+      <c r="A11" s="52"/>
+      <c r="B11" s="53"/>
+      <c r="C11" s="54"/>
       <c r="D11" s="13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E11" s="14"/>
       <c r="F11" s="14"/>
@@ -1387,18 +1388,20 @@
       <c r="Q11" s="15"/>
       <c r="R11" s="15"/>
     </row>
-    <row r="12" spans="1:18" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="56"/>
-      <c r="B12" s="57"/>
-      <c r="C12" s="58"/>
-      <c r="D12" s="59"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="60"/>
-      <c r="I12" s="60"/>
-      <c r="J12" s="60"/>
-      <c r="K12" s="61"/>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A12" s="52"/>
+      <c r="B12" s="53"/>
+      <c r="C12" s="54"/>
+      <c r="D12" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="14"/>
+      <c r="F12" s="14"/>
+      <c r="G12" s="14"/>
+      <c r="H12" s="14"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="14"/>
       <c r="L12" s="6"/>
       <c r="M12" s="15"/>
       <c r="N12" s="12"/>
@@ -1408,11 +1411,11 @@
       <c r="R12" s="15"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A13" s="56"/>
-      <c r="B13" s="57"/>
-      <c r="C13" s="58"/>
+      <c r="A13" s="52"/>
+      <c r="B13" s="53"/>
+      <c r="C13" s="54"/>
       <c r="D13" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E13" s="25"/>
       <c r="F13" s="25"/>
@@ -1430,19 +1433,19 @@
       <c r="R13" s="15"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A14" s="56"/>
-      <c r="B14" s="57"/>
-      <c r="C14" s="58"/>
+      <c r="A14" s="52"/>
+      <c r="B14" s="53"/>
+      <c r="C14" s="54"/>
       <c r="D14" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
+        <v>9</v>
+      </c>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
       <c r="G14" s="14"/>
       <c r="H14" s="14"/>
       <c r="I14" s="14"/>
       <c r="J14" s="14"/>
-      <c r="K14" s="25"/>
+      <c r="K14" s="14"/>
       <c r="L14" s="6"/>
       <c r="M14" s="15"/>
       <c r="N14" s="12"/>
@@ -1452,18 +1455,16 @@
       <c r="R14" s="15"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A15" s="56"/>
-      <c r="B15" s="57"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="25"/>
-      <c r="J15" s="25"/>
+      <c r="A15" s="52"/>
+      <c r="B15" s="53"/>
+      <c r="C15" s="54"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="14"/>
+      <c r="H15" s="14"/>
+      <c r="I15" s="14"/>
+      <c r="J15" s="14"/>
       <c r="K15" s="14"/>
       <c r="L15" s="6"/>
       <c r="M15" s="15"/>
@@ -1473,20 +1474,18 @@
       <c r="Q15" s="15"/>
       <c r="R15" s="15"/>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A16" s="56"/>
-      <c r="B16" s="57"/>
-      <c r="C16" s="58"/>
-      <c r="D16" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
-      <c r="I16" s="25"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="14"/>
+    <row r="16" spans="1:18" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="52"/>
+      <c r="B16" s="53"/>
+      <c r="C16" s="54"/>
+      <c r="D16" s="55"/>
+      <c r="E16" s="56"/>
+      <c r="F16" s="56"/>
+      <c r="G16" s="56"/>
+      <c r="H16" s="56"/>
+      <c r="I16" s="56"/>
+      <c r="J16" s="56"/>
+      <c r="K16" s="57"/>
       <c r="L16" s="6"/>
       <c r="M16" s="15"/>
       <c r="N16" s="12"/>
@@ -1496,19 +1495,19 @@
       <c r="R16" s="15"/>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A17" s="56"/>
-      <c r="B17" s="57"/>
-      <c r="C17" s="58"/>
+      <c r="A17" s="52"/>
+      <c r="B17" s="53"/>
+      <c r="C17" s="54"/>
       <c r="D17" s="13" t="s">
-        <v>48</v>
+        <v>18</v>
       </c>
       <c r="E17" s="14"/>
       <c r="F17" s="14"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="25"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+      <c r="I17" s="14"/>
+      <c r="J17" s="14"/>
+      <c r="K17" s="25"/>
       <c r="L17" s="6"/>
       <c r="M17" s="15"/>
       <c r="N17" s="12"/>
@@ -1518,18 +1517,18 @@
       <c r="R17" s="15"/>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A18" s="56"/>
-      <c r="B18" s="57"/>
-      <c r="C18" s="58"/>
+      <c r="A18" s="52"/>
+      <c r="B18" s="53"/>
+      <c r="C18" s="54"/>
       <c r="D18" s="13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E18" s="14"/>
       <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="25"/>
       <c r="I18" s="25"/>
-      <c r="J18" s="14"/>
+      <c r="J18" s="25"/>
       <c r="K18" s="14"/>
       <c r="L18" s="6"/>
       <c r="M18" s="15"/>
@@ -1539,18 +1538,20 @@
       <c r="Q18" s="15"/>
       <c r="R18" s="15"/>
     </row>
-    <row r="19" spans="1:18" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="56"/>
-      <c r="B19" s="57"/>
-      <c r="C19" s="58"/>
-      <c r="D19" s="59"/>
-      <c r="E19" s="60"/>
-      <c r="F19" s="60"/>
-      <c r="G19" s="60"/>
-      <c r="H19" s="60"/>
-      <c r="I19" s="60"/>
-      <c r="J19" s="60"/>
-      <c r="K19" s="61"/>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A19" s="52"/>
+      <c r="B19" s="53"/>
+      <c r="C19" s="54"/>
+      <c r="D19" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="25"/>
+      <c r="H19" s="25"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="25"/>
+      <c r="K19" s="14"/>
       <c r="L19" s="6"/>
       <c r="M19" s="15"/>
       <c r="N19" s="12"/>
@@ -1560,18 +1561,18 @@
       <c r="R19" s="15"/>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A20" s="56"/>
-      <c r="B20" s="57"/>
-      <c r="C20" s="58"/>
+      <c r="A20" s="52"/>
+      <c r="B20" s="53"/>
+      <c r="C20" s="54"/>
       <c r="D20" s="13" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="E20" s="14"/>
       <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="14"/>
+      <c r="G20" s="25"/>
+      <c r="H20" s="25"/>
+      <c r="I20" s="25"/>
+      <c r="J20" s="25"/>
       <c r="K20" s="14"/>
       <c r="L20" s="6"/>
       <c r="M20" s="15"/>
@@ -1582,19 +1583,19 @@
       <c r="R20" s="15"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A21" s="56"/>
-      <c r="B21" s="57"/>
-      <c r="C21" s="58"/>
+      <c r="A21" s="52"/>
+      <c r="B21" s="53"/>
+      <c r="C21" s="54"/>
       <c r="D21" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="E21" s="17"/>
+        <v>19</v>
+      </c>
+      <c r="E21" s="14"/>
       <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14"/>
-      <c r="K21" s="17"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="25"/>
+      <c r="I21" s="25"/>
+      <c r="J21" s="25"/>
+      <c r="K21" s="14"/>
       <c r="L21" s="6"/>
       <c r="M21" s="15"/>
       <c r="N21" s="12"/>
@@ -1604,18 +1605,16 @@
       <c r="R21" s="15"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A22" s="56"/>
-      <c r="B22" s="57"/>
-      <c r="C22" s="58"/>
-      <c r="D22" s="13" t="s">
-        <v>50</v>
-      </c>
+      <c r="A22" s="52"/>
+      <c r="B22" s="53"/>
+      <c r="C22" s="54"/>
+      <c r="D22" s="13"/>
       <c r="E22" s="14"/>
       <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="14"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="25"/>
+      <c r="I22" s="25"/>
+      <c r="J22" s="25"/>
       <c r="K22" s="14"/>
       <c r="L22" s="6"/>
       <c r="M22" s="15"/>
@@ -1625,18 +1624,20 @@
       <c r="Q22" s="15"/>
       <c r="R22" s="15"/>
     </row>
-    <row r="23" spans="1:18" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
-      <c r="K23" s="6"/>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A23" s="52"/>
+      <c r="B23" s="53"/>
+      <c r="C23" s="54"/>
+      <c r="D23" s="41" t="s">
+        <v>53</v>
+      </c>
+      <c r="E23" s="42"/>
+      <c r="F23" s="42"/>
+      <c r="G23" s="42"/>
+      <c r="H23" s="42"/>
+      <c r="I23" s="43"/>
+      <c r="J23" s="42"/>
+      <c r="K23" s="42"/>
       <c r="L23" s="6"/>
       <c r="M23" s="15"/>
       <c r="N23" s="12"/>
@@ -1645,22 +1646,18 @@
       <c r="Q23" s="15"/>
       <c r="R23" s="15"/>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A24" s="51" t="s">
-        <v>24</v>
-      </c>
-      <c r="B24" s="51"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="E24" s="50"/>
-      <c r="F24" s="50"/>
-      <c r="G24" s="50"/>
-      <c r="H24" s="50"/>
-      <c r="I24" s="50"/>
-      <c r="J24" s="50"/>
-      <c r="K24" s="50"/>
+    <row r="24" spans="1:18" ht="3.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="52"/>
+      <c r="B24" s="53"/>
+      <c r="C24" s="54"/>
+      <c r="D24" s="55"/>
+      <c r="E24" s="56"/>
+      <c r="F24" s="56"/>
+      <c r="G24" s="56"/>
+      <c r="H24" s="56"/>
+      <c r="I24" s="56"/>
+      <c r="J24" s="56"/>
+      <c r="K24" s="57"/>
       <c r="L24" s="6"/>
       <c r="M24" s="15"/>
       <c r="N24" s="12"/>
@@ -1670,11 +1667,11 @@
       <c r="R24" s="15"/>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A25" s="51"/>
-      <c r="B25" s="51"/>
-      <c r="C25" s="51"/>
-      <c r="D25" s="14" t="s">
-        <v>25</v>
+      <c r="A25" s="52"/>
+      <c r="B25" s="53"/>
+      <c r="C25" s="54"/>
+      <c r="D25" s="13" t="s">
+        <v>20</v>
       </c>
       <c r="E25" s="14"/>
       <c r="F25" s="14"/>
@@ -1684,41 +1681,41 @@
       <c r="J25" s="14"/>
       <c r="K25" s="14"/>
       <c r="L25" s="6"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="15"/>
+      <c r="M25" s="15"/>
+      <c r="N25" s="12"/>
       <c r="O25" s="15"/>
       <c r="P25" s="15"/>
       <c r="Q25" s="15"/>
       <c r="R25" s="15"/>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A26" s="51"/>
-      <c r="B26" s="51"/>
-      <c r="C26" s="51"/>
-      <c r="D26" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="E26" s="14"/>
+      <c r="A26" s="52"/>
+      <c r="B26" s="53"/>
+      <c r="C26" s="54"/>
+      <c r="D26" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E26" s="17"/>
       <c r="F26" s="14"/>
       <c r="G26" s="14"/>
       <c r="H26" s="14"/>
       <c r="I26" s="14"/>
       <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
+      <c r="K26" s="17"/>
       <c r="L26" s="6"/>
-      <c r="M26" s="16"/>
-      <c r="N26" s="15"/>
+      <c r="M26" s="15"/>
+      <c r="N26" s="12"/>
       <c r="O26" s="15"/>
       <c r="P26" s="15"/>
       <c r="Q26" s="15"/>
       <c r="R26" s="15"/>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A27" s="51"/>
-      <c r="B27" s="51"/>
-      <c r="C27" s="51"/>
-      <c r="D27" s="14" t="s">
-        <v>26</v>
+      <c r="A27" s="52"/>
+      <c r="B27" s="53"/>
+      <c r="C27" s="54"/>
+      <c r="D27" s="13" t="s">
+        <v>14</v>
       </c>
       <c r="E27" s="14"/>
       <c r="F27" s="14"/>
@@ -1728,63 +1725,63 @@
       <c r="J27" s="14"/>
       <c r="K27" s="14"/>
       <c r="L27" s="6"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="15"/>
+      <c r="M27" s="15"/>
+      <c r="N27" s="12"/>
       <c r="O27" s="15"/>
       <c r="P27" s="15"/>
       <c r="Q27" s="15"/>
       <c r="R27" s="15"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A28" s="51"/>
-      <c r="B28" s="51"/>
-      <c r="C28" s="51"/>
-      <c r="D28" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="E28" s="14"/>
+    <row r="28" spans="1:18" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
       <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="14"/>
-      <c r="J28" s="14"/>
-      <c r="K28" s="14"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="6"/>
+      <c r="K28" s="6"/>
       <c r="L28" s="6"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="15"/>
+      <c r="M28" s="15"/>
+      <c r="N28" s="12"/>
       <c r="O28" s="15"/>
       <c r="P28" s="15"/>
       <c r="Q28" s="15"/>
       <c r="R28" s="15"/>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A29" s="51"/>
-      <c r="B29" s="51"/>
-      <c r="C29" s="51"/>
+      <c r="A29" s="47" t="s">
+        <v>23</v>
+      </c>
+      <c r="B29" s="47"/>
+      <c r="C29" s="47"/>
       <c r="D29" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="14"/>
-      <c r="I29" s="14"/>
-      <c r="J29" s="14"/>
-      <c r="K29" s="14"/>
+        <v>26</v>
+      </c>
+      <c r="E29" s="40"/>
+      <c r="F29" s="40"/>
+      <c r="G29" s="40"/>
+      <c r="H29" s="40"/>
+      <c r="I29" s="40"/>
+      <c r="J29" s="40"/>
+      <c r="K29" s="40"/>
       <c r="L29" s="6"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="15"/>
+      <c r="M29" s="15"/>
+      <c r="N29" s="12"/>
       <c r="O29" s="15"/>
       <c r="P29" s="15"/>
       <c r="Q29" s="15"/>
       <c r="R29" s="15"/>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A30" s="51"/>
-      <c r="B30" s="51"/>
-      <c r="C30" s="51"/>
+      <c r="A30" s="47"/>
+      <c r="B30" s="47"/>
+      <c r="C30" s="47"/>
       <c r="D30" s="14" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="E30" s="14"/>
       <c r="F30" s="14"/>
@@ -1802,11 +1799,11 @@
       <c r="R30" s="15"/>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A31" s="51"/>
-      <c r="B31" s="51"/>
-      <c r="C31" s="51"/>
+      <c r="A31" s="47"/>
+      <c r="B31" s="47"/>
+      <c r="C31" s="47"/>
       <c r="D31" s="14" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
       <c r="E31" s="14"/>
       <c r="F31" s="14"/>
@@ -1824,11 +1821,11 @@
       <c r="R31" s="15"/>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A32" s="51"/>
-      <c r="B32" s="51"/>
-      <c r="C32" s="51"/>
+      <c r="A32" s="47"/>
+      <c r="B32" s="47"/>
+      <c r="C32" s="47"/>
       <c r="D32" s="14" t="s">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="E32" s="14"/>
       <c r="F32" s="14"/>
@@ -1846,11 +1843,11 @@
       <c r="R32" s="15"/>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A33" s="51"/>
-      <c r="B33" s="51"/>
-      <c r="C33" s="51"/>
+      <c r="A33" s="47"/>
+      <c r="B33" s="47"/>
+      <c r="C33" s="47"/>
       <c r="D33" s="14" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E33" s="14"/>
       <c r="F33" s="14"/>
@@ -1868,11 +1865,11 @@
       <c r="R33" s="15"/>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A34" s="51"/>
-      <c r="B34" s="51"/>
-      <c r="C34" s="51"/>
+      <c r="A34" s="47"/>
+      <c r="B34" s="47"/>
+      <c r="C34" s="47"/>
       <c r="D34" s="14" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E34" s="14"/>
       <c r="F34" s="14"/>
@@ -1890,11 +1887,11 @@
       <c r="R34" s="15"/>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A35" s="51"/>
-      <c r="B35" s="51"/>
-      <c r="C35" s="51"/>
+      <c r="A35" s="47"/>
+      <c r="B35" s="47"/>
+      <c r="C35" s="47"/>
       <c r="D35" s="14" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="E35" s="14"/>
       <c r="F35" s="14"/>
@@ -1911,34 +1908,34 @@
       <c r="Q35" s="15"/>
       <c r="R35" s="15"/>
     </row>
-    <row r="36" spans="1:18" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="1"/>
-      <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="18"/>
-      <c r="I36" s="5"/>
-      <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
-      <c r="L36" s="5"/>
-      <c r="M36" s="19"/>
-      <c r="N36" s="20"/>
-      <c r="O36" s="16"/>
-      <c r="P36" s="16"/>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A36" s="47"/>
+      <c r="B36" s="47"/>
+      <c r="C36" s="47"/>
+      <c r="D36" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
+      <c r="I36" s="14"/>
+      <c r="J36" s="14"/>
+      <c r="K36" s="14"/>
+      <c r="L36" s="6"/>
+      <c r="M36" s="16"/>
+      <c r="N36" s="15"/>
+      <c r="O36" s="15"/>
+      <c r="P36" s="15"/>
       <c r="Q36" s="15"/>
       <c r="R36" s="15"/>
     </row>
-    <row r="37" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="51" t="s">
-        <v>31</v>
-      </c>
-      <c r="B37" s="51"/>
-      <c r="C37" s="51"/>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A37" s="47"/>
+      <c r="B37" s="47"/>
+      <c r="C37" s="47"/>
       <c r="D37" s="14" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="E37" s="14"/>
       <c r="F37" s="14"/>
@@ -1947,21 +1944,19 @@
       <c r="I37" s="14"/>
       <c r="J37" s="14"/>
       <c r="K37" s="14"/>
-      <c r="L37" s="5"/>
-      <c r="M37" s="19"/>
-      <c r="N37" s="20"/>
-      <c r="O37" s="16"/>
-      <c r="P37" s="16"/>
+      <c r="L37" s="6"/>
+      <c r="M37" s="16"/>
+      <c r="N37" s="15"/>
+      <c r="O37" s="15"/>
+      <c r="P37" s="15"/>
       <c r="Q37" s="15"/>
       <c r="R37" s="15"/>
     </row>
-    <row r="38" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="51"/>
-      <c r="B38" s="51"/>
-      <c r="C38" s="51"/>
-      <c r="D38" s="14" t="s">
-        <v>33</v>
-      </c>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A38" s="47"/>
+      <c r="B38" s="47"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="14"/>
       <c r="E38" s="14"/>
       <c r="F38" s="14"/>
       <c r="G38" s="14"/>
@@ -1969,76 +1964,72 @@
       <c r="I38" s="14"/>
       <c r="J38" s="14"/>
       <c r="K38" s="14"/>
-      <c r="L38" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="M38" s="19"/>
-      <c r="N38" s="20"/>
-      <c r="O38" s="16"/>
-      <c r="P38" s="16"/>
+      <c r="L38" s="6"/>
+      <c r="M38" s="16"/>
+      <c r="N38" s="15"/>
+      <c r="O38" s="15"/>
+      <c r="P38" s="15"/>
       <c r="Q38" s="15"/>
       <c r="R38" s="15"/>
     </row>
-    <row r="39" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="51"/>
-      <c r="B39" s="51"/>
-      <c r="C39" s="51"/>
-      <c r="D39" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E39" s="14"/>
-      <c r="F39" s="17"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="14"/>
-      <c r="J39" s="17"/>
-      <c r="K39" s="17"/>
-      <c r="L39" s="5"/>
-      <c r="M39" s="19"/>
-      <c r="N39" s="20"/>
-      <c r="O39" s="16"/>
-      <c r="P39" s="16"/>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A39" s="47"/>
+      <c r="B39" s="47"/>
+      <c r="C39" s="47"/>
+      <c r="D39" s="44" t="s">
+        <v>58</v>
+      </c>
+      <c r="E39" s="44"/>
+      <c r="F39" s="44"/>
+      <c r="G39" s="44"/>
+      <c r="H39" s="44"/>
+      <c r="I39" s="44"/>
+      <c r="J39" s="44"/>
+      <c r="K39" s="44"/>
+      <c r="L39" s="6"/>
+      <c r="M39" s="16"/>
+      <c r="N39" s="15"/>
+      <c r="O39" s="15"/>
+      <c r="P39" s="15"/>
       <c r="Q39" s="15"/>
       <c r="R39" s="15"/>
     </row>
-    <row r="40" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="51"/>
-      <c r="B40" s="51"/>
-      <c r="C40" s="51"/>
-      <c r="D40" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="E40" s="14"/>
-      <c r="F40" s="17"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="14"/>
-      <c r="J40" s="17"/>
-      <c r="K40" s="17"/>
-      <c r="L40" s="5"/>
-      <c r="M40" s="19"/>
-      <c r="N40" s="20"/>
-      <c r="O40" s="16"/>
-      <c r="P40" s="16"/>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A40" s="47"/>
+      <c r="B40" s="47"/>
+      <c r="C40" s="47"/>
+      <c r="D40" s="42" t="s">
+        <v>59</v>
+      </c>
+      <c r="E40" s="42"/>
+      <c r="F40" s="42"/>
+      <c r="G40" s="42"/>
+      <c r="H40" s="42"/>
+      <c r="I40" s="42"/>
+      <c r="J40" s="42"/>
+      <c r="K40" s="42"/>
+      <c r="L40" s="6"/>
+      <c r="M40" s="16"/>
+      <c r="N40" s="15"/>
+      <c r="O40" s="15"/>
+      <c r="P40" s="15"/>
       <c r="Q40" s="15"/>
       <c r="R40" s="15"/>
     </row>
-    <row r="41" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="51"/>
-      <c r="B41" s="51"/>
-      <c r="C41" s="51"/>
-      <c r="D41" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="E41" s="17"/>
-      <c r="F41" s="14"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="14"/>
-      <c r="I41" s="17"/>
-      <c r="J41" s="14"/>
-      <c r="K41" s="14"/>
-      <c r="L41" s="6"/>
-      <c r="M41" s="21"/>
+    <row r="41" spans="1:18" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="1"/>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
+      <c r="D41" s="5"/>
+      <c r="E41" s="5"/>
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="18"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="5"/>
+      <c r="K41" s="5"/>
+      <c r="L41" s="5"/>
+      <c r="M41" s="19"/>
       <c r="N41" s="20"/>
       <c r="O41" s="16"/>
       <c r="P41" s="16"/>
@@ -2046,40 +2037,46 @@
       <c r="R41" s="15"/>
     </row>
     <row r="42" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="51"/>
-      <c r="B42" s="51"/>
-      <c r="C42" s="51"/>
+      <c r="A42" s="47" t="s">
+        <v>30</v>
+      </c>
+      <c r="B42" s="47"/>
+      <c r="C42" s="47"/>
       <c r="D42" s="14" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E42" s="14"/>
       <c r="F42" s="14"/>
       <c r="G42" s="14"/>
-      <c r="H42" s="17"/>
+      <c r="H42" s="14"/>
       <c r="I42" s="14"/>
       <c r="J42" s="14"/>
       <c r="K42" s="14"/>
-      <c r="L42" s="6"/>
-      <c r="M42" s="21"/>
+      <c r="L42" s="5"/>
+      <c r="M42" s="19"/>
       <c r="N42" s="20"/>
       <c r="O42" s="16"/>
       <c r="P42" s="16"/>
       <c r="Q42" s="15"/>
       <c r="R42" s="15"/>
     </row>
-    <row r="43" spans="1:18" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="1"/>
-      <c r="B43" s="1"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="6"/>
-      <c r="E43" s="6"/>
-      <c r="F43" s="6"/>
-      <c r="G43" s="6"/>
-      <c r="H43" s="6"/>
-      <c r="I43" s="6"/>
-      <c r="J43" s="6"/>
-      <c r="K43" s="6"/>
-      <c r="L43" s="5"/>
+    <row r="43" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="47"/>
+      <c r="B43" s="47"/>
+      <c r="C43" s="47"/>
+      <c r="D43" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+      <c r="G43" s="14"/>
+      <c r="H43" s="14"/>
+      <c r="I43" s="14"/>
+      <c r="J43" s="14"/>
+      <c r="K43" s="14"/>
+      <c r="L43" s="5" t="s">
+        <v>33</v>
+      </c>
       <c r="M43" s="19"/>
       <c r="N43" s="20"/>
       <c r="O43" s="16"/>
@@ -2088,241 +2085,200 @@
       <c r="R43" s="15"/>
     </row>
     <row r="44" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="64" t="s">
+      <c r="A44" s="47"/>
+      <c r="B44" s="47"/>
+      <c r="C44" s="47"/>
+      <c r="D44" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E44" s="14"/>
+      <c r="F44" s="17"/>
+      <c r="G44" s="14"/>
+      <c r="H44" s="14"/>
+      <c r="I44" s="14"/>
+      <c r="J44" s="17"/>
+      <c r="K44" s="17"/>
+      <c r="L44" s="5"/>
+      <c r="M44" s="19"/>
+      <c r="N44" s="20"/>
+      <c r="O44" s="16"/>
+      <c r="P44" s="16"/>
+      <c r="Q44" s="15"/>
+      <c r="R44" s="15"/>
+    </row>
+    <row r="45" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="47"/>
+      <c r="B45" s="47"/>
+      <c r="C45" s="47"/>
+      <c r="D45" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="E45" s="14"/>
+      <c r="F45" s="17"/>
+      <c r="G45" s="14"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="14"/>
+      <c r="J45" s="17"/>
+      <c r="K45" s="17"/>
+      <c r="L45" s="5"/>
+      <c r="M45" s="19"/>
+      <c r="N45" s="20"/>
+      <c r="O45" s="16"/>
+      <c r="P45" s="16"/>
+      <c r="Q45" s="15"/>
+      <c r="R45" s="15"/>
+    </row>
+    <row r="46" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="47"/>
+      <c r="B46" s="47"/>
+      <c r="C46" s="47"/>
+      <c r="D46" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E46" s="17"/>
+      <c r="F46" s="14"/>
+      <c r="G46" s="17"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="17"/>
+      <c r="J46" s="14"/>
+      <c r="K46" s="14"/>
+      <c r="L46" s="6"/>
+      <c r="M46" s="21"/>
+      <c r="N46" s="20"/>
+      <c r="O46" s="16"/>
+      <c r="P46" s="16"/>
+      <c r="Q46" s="15"/>
+      <c r="R46" s="15"/>
+    </row>
+    <row r="47" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="47"/>
+      <c r="B47" s="47"/>
+      <c r="C47" s="47"/>
+      <c r="D47" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="E47" s="14"/>
+      <c r="F47" s="14"/>
+      <c r="G47" s="14"/>
+      <c r="H47" s="17"/>
+      <c r="I47" s="14"/>
+      <c r="J47" s="14"/>
+      <c r="K47" s="14"/>
+      <c r="L47" s="6"/>
+      <c r="M47" s="21"/>
+      <c r="N47" s="20"/>
+      <c r="O47" s="16"/>
+      <c r="P47" s="16"/>
+      <c r="Q47" s="15"/>
+      <c r="R47" s="15"/>
+    </row>
+    <row r="48" spans="1:18" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="1"/>
+      <c r="B48" s="1"/>
+      <c r="C48" s="1"/>
+      <c r="D48" s="6"/>
+      <c r="E48" s="6"/>
+      <c r="F48" s="6"/>
+      <c r="G48" s="6"/>
+      <c r="H48" s="6"/>
+      <c r="I48" s="6"/>
+      <c r="J48" s="6"/>
+      <c r="K48" s="6"/>
+      <c r="L48" s="5"/>
+      <c r="M48" s="19"/>
+      <c r="N48" s="20"/>
+      <c r="O48" s="16"/>
+      <c r="P48" s="16"/>
+      <c r="Q48" s="15"/>
+      <c r="R48" s="15"/>
+    </row>
+    <row r="49" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="58" t="s">
+        <v>37</v>
+      </c>
+      <c r="B49" s="58"/>
+      <c r="C49" s="58"/>
+      <c r="D49" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B44" s="64"/>
-      <c r="C44" s="64"/>
-      <c r="D44" s="17" t="s">
+      <c r="E49" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="E44" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="F44" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="G44" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="H44" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="I44" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="J44" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="K44" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="L44" s="5"/>
-      <c r="M44" s="12"/>
-      <c r="N44" s="15"/>
-      <c r="O44" s="20"/>
-      <c r="P44" s="23"/>
-      <c r="Q44" s="19"/>
-      <c r="R44" s="19"/>
-    </row>
-    <row r="45" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="65"/>
-      <c r="B45" s="65"/>
-      <c r="C45" s="65"/>
-      <c r="D45" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="E45" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="F45" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="G45" s="22" t="s">
-        <v>42</v>
-      </c>
-      <c r="H45" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="I45" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="J45" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="K45" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="L45" s="5"/>
-      <c r="M45" s="12"/>
-      <c r="N45" s="15"/>
-      <c r="O45" s="20"/>
-      <c r="P45" s="23"/>
-      <c r="Q45" s="19"/>
-      <c r="R45" s="19"/>
-    </row>
-    <row r="46" spans="1:18" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="1"/>
-      <c r="B46" s="1"/>
-      <c r="C46" s="1"/>
-      <c r="D46" s="5"/>
-      <c r="E46" s="5"/>
-      <c r="F46" s="5"/>
-      <c r="G46" s="6"/>
-      <c r="H46" s="5"/>
-      <c r="I46" s="5"/>
-      <c r="J46" s="5"/>
-      <c r="K46" s="5"/>
-      <c r="L46" s="5"/>
-      <c r="M46" s="12"/>
-      <c r="N46" s="15"/>
-      <c r="O46" s="12"/>
-      <c r="P46" s="12"/>
-      <c r="Q46" s="12"/>
-      <c r="R46" s="12"/>
-    </row>
-    <row r="47" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="66" t="s">
-        <v>43</v>
-      </c>
-      <c r="B47" s="67"/>
-      <c r="C47" s="68"/>
-      <c r="D47" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="E47" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="F47" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="G47" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="H47" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="I47" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="J47" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="K47" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="L47" s="5"/>
-      <c r="M47" s="12"/>
-      <c r="N47" s="15"/>
-      <c r="O47" s="12"/>
-      <c r="P47" s="12"/>
-      <c r="Q47" s="12"/>
-      <c r="R47" s="12"/>
-    </row>
-    <row r="48" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="69"/>
-      <c r="B48" s="70"/>
-      <c r="C48" s="71"/>
-      <c r="D48" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="E48" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="F48" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="G48" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="H48" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="I48" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="J48" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="K48" s="25" t="s">
-        <v>45</v>
-      </c>
-      <c r="L48" s="5"/>
-      <c r="M48" s="12"/>
-      <c r="N48" s="15"/>
-      <c r="O48" s="12"/>
-      <c r="P48" s="12"/>
-      <c r="Q48" s="12"/>
-      <c r="R48" s="12"/>
-    </row>
-    <row r="49" spans="1:18" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="1"/>
-      <c r="B49" s="1"/>
-      <c r="C49" s="1"/>
-      <c r="D49" s="26"/>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
-      <c r="G49" s="6"/>
-      <c r="H49" s="5"/>
-      <c r="I49" s="5"/>
-      <c r="J49" s="5"/>
-      <c r="K49" s="5"/>
+      <c r="F49" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="G49" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="H49" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="I49" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="J49" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="K49" s="22" t="s">
+        <v>39</v>
+      </c>
       <c r="L49" s="5"/>
       <c r="M49" s="12"/>
       <c r="N49" s="15"/>
-      <c r="O49" s="12"/>
-      <c r="P49" s="12"/>
-      <c r="Q49" s="12"/>
-      <c r="R49" s="12"/>
+      <c r="O49" s="20"/>
+      <c r="P49" s="23"/>
+      <c r="Q49" s="19"/>
+      <c r="R49" s="19"/>
     </row>
     <row r="50" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="72" t="s">
-        <v>46</v>
-      </c>
-      <c r="B50" s="73"/>
-      <c r="C50" s="74"/>
-      <c r="D50" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="E50" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="F50" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="G50" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="H50" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="I50" s="25" t="s">
-        <v>14</v>
-      </c>
-      <c r="J50" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="K50" s="14" t="s">
-        <v>14</v>
+      <c r="A50" s="59"/>
+      <c r="B50" s="59"/>
+      <c r="C50" s="59"/>
+      <c r="D50" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E50" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="G50" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="H50" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="I50" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="J50" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="K50" s="24" t="s">
+        <v>13</v>
       </c>
       <c r="L50" s="5"/>
       <c r="M50" s="12"/>
       <c r="N50" s="15"/>
-      <c r="O50" s="12"/>
-      <c r="P50" s="12"/>
-      <c r="Q50" s="12"/>
-      <c r="R50" s="12"/>
-    </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D51" s="27"/>
-      <c r="E51" s="28"/>
-      <c r="F51" s="28"/>
-      <c r="G51" s="29"/>
-      <c r="H51" s="28"/>
-      <c r="I51" s="28"/>
-      <c r="J51" s="28"/>
-      <c r="K51" s="28"/>
-      <c r="L51" s="42"/>
+      <c r="O50" s="20"/>
+      <c r="P50" s="23"/>
+      <c r="Q50" s="19"/>
+      <c r="R50" s="19"/>
+    </row>
+    <row r="51" spans="1:18" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="1"/>
+      <c r="B51" s="1"/>
+      <c r="C51" s="1"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="6"/>
+      <c r="H51" s="5"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="K51" s="5"/>
+      <c r="L51" s="5"/>
       <c r="M51" s="12"/>
       <c r="N51" s="15"/>
       <c r="O51" s="12"/>
@@ -2330,16 +2286,37 @@
       <c r="Q51" s="12"/>
       <c r="R51" s="12"/>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D52" s="30"/>
-      <c r="E52" s="31"/>
-      <c r="F52" s="31"/>
-      <c r="G52" s="32"/>
-      <c r="H52" s="31"/>
-      <c r="I52" s="31"/>
-      <c r="J52" s="31"/>
-      <c r="K52" s="31"/>
-      <c r="L52" s="42"/>
+    <row r="52" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="60" t="s">
+        <v>42</v>
+      </c>
+      <c r="B52" s="61"/>
+      <c r="C52" s="62"/>
+      <c r="D52" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="E52" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="F52" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="G52" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="H52" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="I52" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="J52" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="K52" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="L52" s="5"/>
       <c r="M52" s="12"/>
       <c r="N52" s="15"/>
       <c r="O52" s="12"/>
@@ -2347,317 +2324,442 @@
       <c r="Q52" s="12"/>
       <c r="R52" s="12"/>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D53" s="75"/>
-      <c r="E53" s="75"/>
-      <c r="F53" s="75"/>
-      <c r="G53" s="75"/>
-      <c r="H53" s="75"/>
-      <c r="I53" s="75"/>
-      <c r="J53" s="75"/>
-      <c r="K53" s="75"/>
-      <c r="L53" s="43"/>
-      <c r="M53" s="19"/>
-      <c r="N53" s="19"/>
+    <row r="53" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="63"/>
+      <c r="B53" s="64"/>
+      <c r="C53" s="65"/>
+      <c r="D53" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="E53" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="F53" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="G53" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="H53" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="I53" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="J53" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="K53" s="25" t="s">
+        <v>44</v>
+      </c>
+      <c r="L53" s="5"/>
+      <c r="M53" s="12"/>
+      <c r="N53" s="15"/>
       <c r="O53" s="12"/>
       <c r="P53" s="12"/>
       <c r="Q53" s="12"/>
       <c r="R53" s="12"/>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D54" s="62"/>
-      <c r="E54" s="62"/>
-      <c r="F54" s="62"/>
-      <c r="G54" s="62"/>
-      <c r="H54" s="62"/>
-      <c r="I54" s="62"/>
-      <c r="J54" s="62"/>
-      <c r="K54" s="62"/>
-      <c r="L54" s="45"/>
-      <c r="M54" s="8"/>
-      <c r="N54" s="8"/>
-      <c r="O54" s="19"/>
-      <c r="P54" s="19"/>
-      <c r="Q54" s="19"/>
-      <c r="R54" s="19"/>
-    </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D55" s="62"/>
-      <c r="E55" s="62"/>
-      <c r="F55" s="62"/>
-      <c r="G55" s="62"/>
-      <c r="H55" s="62"/>
-      <c r="I55" s="62"/>
-      <c r="J55" s="62"/>
-      <c r="K55" s="62"/>
-      <c r="L55" s="45"/>
-      <c r="M55" s="8"/>
-      <c r="N55" s="8"/>
-      <c r="O55" s="8"/>
-      <c r="P55" s="8"/>
-      <c r="Q55" s="8"/>
-      <c r="R55" s="8"/>
+    <row r="54" spans="1:18" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="1"/>
+      <c r="B54" s="1"/>
+      <c r="C54" s="1"/>
+      <c r="D54" s="26"/>
+      <c r="E54" s="5"/>
+      <c r="F54" s="5"/>
+      <c r="G54" s="6"/>
+      <c r="H54" s="5"/>
+      <c r="I54" s="5"/>
+      <c r="J54" s="5"/>
+      <c r="K54" s="5"/>
+      <c r="L54" s="5"/>
+      <c r="M54" s="12"/>
+      <c r="N54" s="15"/>
+      <c r="O54" s="12"/>
+      <c r="P54" s="12"/>
+      <c r="Q54" s="12"/>
+      <c r="R54" s="12"/>
+    </row>
+    <row r="55" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="66" t="s">
+        <v>45</v>
+      </c>
+      <c r="B55" s="67"/>
+      <c r="C55" s="68"/>
+      <c r="D55" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="E55" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="F55" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="G55" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="H55" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="I55" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="J55" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="K55" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="L55" s="5"/>
+      <c r="M55" s="12"/>
+      <c r="N55" s="15"/>
+      <c r="O55" s="12"/>
+      <c r="P55" s="12"/>
+      <c r="Q55" s="12"/>
+      <c r="R55" s="12"/>
     </row>
     <row r="56" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D56" s="44"/>
-      <c r="E56" s="46"/>
-      <c r="F56" s="46"/>
-      <c r="G56" s="46"/>
-      <c r="H56" s="46"/>
-      <c r="I56" s="46"/>
-      <c r="J56" s="46"/>
-      <c r="K56" s="46"/>
-      <c r="L56" s="46"/>
-      <c r="M56" s="11"/>
-      <c r="N56" s="11"/>
-      <c r="O56" s="11"/>
-      <c r="P56" s="11"/>
-      <c r="Q56" s="11"/>
-      <c r="R56" s="11"/>
+      <c r="D56" s="27"/>
+      <c r="E56" s="28"/>
+      <c r="F56" s="28"/>
+      <c r="G56" s="29"/>
+      <c r="H56" s="28"/>
+      <c r="I56" s="28"/>
+      <c r="J56" s="28"/>
+      <c r="K56" s="28"/>
+      <c r="L56" s="37"/>
+      <c r="M56" s="12"/>
+      <c r="N56" s="15"/>
+      <c r="O56" s="12"/>
+      <c r="P56" s="12"/>
+      <c r="Q56" s="12"/>
+      <c r="R56" s="12"/>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D57" s="63"/>
-      <c r="E57" s="63"/>
-      <c r="F57" s="63"/>
-      <c r="G57" s="63"/>
-      <c r="H57" s="63"/>
-      <c r="I57" s="63"/>
-      <c r="J57" s="63"/>
-      <c r="K57" s="63"/>
-      <c r="L57" s="47"/>
-      <c r="M57" s="15"/>
-      <c r="N57" s="12"/>
-      <c r="O57" s="16"/>
-      <c r="P57" s="16"/>
-      <c r="Q57" s="16"/>
-      <c r="R57" s="16"/>
+      <c r="D57" s="30"/>
+      <c r="E57" s="31"/>
+      <c r="F57" s="31"/>
+      <c r="G57" s="32"/>
+      <c r="H57" s="31"/>
+      <c r="I57" s="31"/>
+      <c r="J57" s="31"/>
+      <c r="K57" s="31"/>
+      <c r="L57" s="37"/>
+      <c r="M57" s="12"/>
+      <c r="N57" s="15"/>
+      <c r="O57" s="12"/>
+      <c r="P57" s="12"/>
+      <c r="Q57" s="12"/>
+      <c r="R57" s="12"/>
     </row>
     <row r="58" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D58" s="27"/>
-      <c r="E58" s="48"/>
-      <c r="F58" s="48"/>
-      <c r="G58" s="49"/>
-      <c r="H58" s="48"/>
-      <c r="I58" s="48"/>
-      <c r="J58" s="48"/>
-      <c r="K58" s="48"/>
-      <c r="L58" s="44"/>
-      <c r="M58" s="15"/>
-      <c r="N58" s="12"/>
-      <c r="O58" s="15"/>
-      <c r="P58" s="15"/>
-      <c r="Q58" s="15"/>
-      <c r="R58" s="15"/>
+      <c r="D58" s="45"/>
+      <c r="E58" s="45"/>
+      <c r="F58" s="45"/>
+      <c r="G58" s="45"/>
+      <c r="H58" s="45"/>
+      <c r="I58" s="45"/>
+      <c r="J58" s="45"/>
+      <c r="K58" s="45"/>
+      <c r="L58" s="38"/>
+      <c r="M58" s="19"/>
+      <c r="N58" s="19"/>
+      <c r="O58" s="12"/>
+      <c r="P58" s="12"/>
+      <c r="Q58" s="12"/>
+      <c r="R58" s="12"/>
     </row>
     <row r="59" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D59" s="33"/>
-      <c r="E59" s="34"/>
-      <c r="F59" s="34"/>
-      <c r="G59" s="35"/>
-      <c r="H59" s="34"/>
-      <c r="I59" s="34"/>
-      <c r="J59" s="34"/>
-      <c r="K59" s="34"/>
-      <c r="L59" s="15"/>
-      <c r="M59" s="15"/>
-      <c r="N59" s="16"/>
-      <c r="O59" s="15"/>
-      <c r="P59" s="15"/>
-      <c r="Q59" s="16"/>
-      <c r="R59" s="16"/>
+      <c r="D59" s="45"/>
+      <c r="E59" s="45"/>
+      <c r="F59" s="45"/>
+      <c r="G59" s="45"/>
+      <c r="H59" s="45"/>
+      <c r="I59" s="45"/>
+      <c r="J59" s="45"/>
+      <c r="K59" s="45"/>
+      <c r="L59" s="39"/>
+      <c r="M59" s="8"/>
+      <c r="N59" s="8"/>
+      <c r="O59" s="19"/>
+      <c r="P59" s="19"/>
+      <c r="Q59" s="19"/>
+      <c r="R59" s="19"/>
     </row>
     <row r="60" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D60" s="33"/>
-      <c r="E60" s="36"/>
-      <c r="F60" s="36"/>
-      <c r="G60" s="37"/>
-      <c r="H60" s="36"/>
-      <c r="I60" s="36"/>
-      <c r="J60" s="36"/>
-      <c r="K60" s="36"/>
-      <c r="L60" s="15"/>
-      <c r="M60" s="15"/>
-      <c r="N60" s="15"/>
-      <c r="O60" s="15"/>
-      <c r="P60" s="16"/>
-      <c r="Q60" s="15"/>
-      <c r="R60" s="15"/>
+      <c r="D60" s="45"/>
+      <c r="E60" s="45"/>
+      <c r="F60" s="45"/>
+      <c r="G60" s="45"/>
+      <c r="H60" s="45"/>
+      <c r="I60" s="45"/>
+      <c r="J60" s="45"/>
+      <c r="K60" s="45"/>
+      <c r="L60" s="39"/>
+      <c r="M60" s="8"/>
+      <c r="N60" s="8"/>
+      <c r="O60" s="8"/>
+      <c r="P60" s="8"/>
+      <c r="Q60" s="8"/>
+      <c r="R60" s="8"/>
     </row>
     <row r="61" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D61" s="16"/>
-      <c r="E61" s="15"/>
-      <c r="F61" s="15"/>
-      <c r="G61" s="15"/>
-      <c r="H61" s="15"/>
-      <c r="I61" s="15"/>
-      <c r="J61" s="15"/>
-      <c r="K61" s="15"/>
-      <c r="L61" s="16"/>
-      <c r="M61" s="16"/>
-      <c r="N61" s="15"/>
-      <c r="O61" s="15"/>
-      <c r="P61" s="15"/>
-      <c r="Q61" s="15"/>
-      <c r="R61" s="15"/>
+      <c r="D61" s="46"/>
+      <c r="E61" s="46"/>
+      <c r="F61" s="46"/>
+      <c r="G61" s="46"/>
+      <c r="H61" s="46"/>
+      <c r="I61" s="46"/>
+      <c r="J61" s="46"/>
+      <c r="K61" s="46"/>
+      <c r="L61" s="46"/>
+      <c r="M61" s="11"/>
+      <c r="N61" s="11"/>
+      <c r="O61" s="11"/>
+      <c r="P61" s="11"/>
+      <c r="Q61" s="11"/>
+      <c r="R61" s="11"/>
     </row>
     <row r="62" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D62" s="16"/>
-      <c r="E62" s="15"/>
-      <c r="F62" s="16"/>
-      <c r="G62" s="15"/>
-      <c r="H62" s="15"/>
-      <c r="I62" s="15"/>
-      <c r="J62" s="15"/>
-      <c r="K62" s="15"/>
-      <c r="L62" s="15"/>
-      <c r="M62" s="16"/>
-      <c r="N62" s="15"/>
-      <c r="O62" s="15"/>
-      <c r="P62" s="15"/>
-      <c r="Q62" s="15"/>
-      <c r="R62" s="15"/>
+      <c r="D62" s="46"/>
+      <c r="E62" s="46"/>
+      <c r="F62" s="46"/>
+      <c r="G62" s="46"/>
+      <c r="H62" s="46"/>
+      <c r="I62" s="46"/>
+      <c r="J62" s="46"/>
+      <c r="K62" s="46"/>
+      <c r="L62" s="46"/>
+      <c r="M62" s="15"/>
+      <c r="N62" s="12"/>
+      <c r="O62" s="16"/>
+      <c r="P62" s="16"/>
+      <c r="Q62" s="16"/>
+      <c r="R62" s="16"/>
     </row>
     <row r="63" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D63" s="16"/>
-      <c r="E63" s="15"/>
-      <c r="F63" s="15"/>
-      <c r="G63" s="15"/>
-      <c r="H63" s="16"/>
-      <c r="I63" s="16"/>
-      <c r="J63" s="15"/>
-      <c r="K63" s="15"/>
-      <c r="L63" s="15"/>
+      <c r="D63" s="46"/>
+      <c r="E63" s="46"/>
+      <c r="F63" s="46"/>
+      <c r="G63" s="46"/>
+      <c r="H63" s="46"/>
+      <c r="I63" s="46"/>
+      <c r="J63" s="46"/>
+      <c r="K63" s="46"/>
+      <c r="L63" s="46"/>
       <c r="M63" s="15"/>
-      <c r="N63" s="15"/>
-      <c r="O63" s="16"/>
-      <c r="P63" s="16"/>
+      <c r="N63" s="12"/>
+      <c r="O63" s="15"/>
+      <c r="P63" s="15"/>
       <c r="Q63" s="15"/>
       <c r="R63" s="15"/>
     </row>
     <row r="64" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="D64" s="16"/>
-      <c r="E64" s="15"/>
-      <c r="F64" s="15"/>
-      <c r="G64" s="15"/>
-      <c r="H64" s="15"/>
-      <c r="I64" s="15"/>
-      <c r="J64" s="15"/>
-      <c r="K64" s="15"/>
-      <c r="L64" s="15"/>
+      <c r="D64" s="46"/>
+      <c r="E64" s="46"/>
+      <c r="F64" s="46"/>
+      <c r="G64" s="46"/>
+      <c r="H64" s="46"/>
+      <c r="I64" s="46"/>
+      <c r="J64" s="46"/>
+      <c r="K64" s="46"/>
+      <c r="L64" s="46"/>
       <c r="M64" s="15"/>
-      <c r="N64" s="15"/>
+      <c r="N64" s="16"/>
       <c r="O64" s="15"/>
       <c r="P64" s="15"/>
-      <c r="Q64" s="15"/>
-      <c r="R64" s="15"/>
+      <c r="Q64" s="16"/>
+      <c r="R64" s="16"/>
     </row>
     <row r="65" spans="4:18" x14ac:dyDescent="0.2">
-      <c r="D65" s="16"/>
-      <c r="E65" s="15"/>
-      <c r="F65" s="15"/>
-      <c r="G65" s="15"/>
-      <c r="H65" s="15"/>
-      <c r="I65" s="15"/>
-      <c r="J65" s="15"/>
-      <c r="K65" s="15"/>
-      <c r="L65" s="15"/>
+      <c r="D65" s="46"/>
+      <c r="E65" s="46"/>
+      <c r="F65" s="46"/>
+      <c r="G65" s="46"/>
+      <c r="H65" s="46"/>
+      <c r="I65" s="46"/>
+      <c r="J65" s="46"/>
+      <c r="K65" s="46"/>
+      <c r="L65" s="46"/>
       <c r="M65" s="15"/>
       <c r="N65" s="15"/>
       <c r="O65" s="15"/>
-      <c r="P65" s="15"/>
+      <c r="P65" s="16"/>
       <c r="Q65" s="15"/>
       <c r="R65" s="15"/>
     </row>
     <row r="66" spans="4:18" x14ac:dyDescent="0.2">
-      <c r="D66" s="38"/>
-      <c r="E66" s="15"/>
-      <c r="F66" s="16"/>
-      <c r="G66" s="16"/>
-      <c r="H66" s="15"/>
-      <c r="I66" s="15"/>
-      <c r="J66" s="15"/>
-      <c r="K66" s="12"/>
-      <c r="L66" s="15"/>
+      <c r="D66" s="46"/>
+      <c r="E66" s="46"/>
+      <c r="F66" s="46"/>
+      <c r="G66" s="46"/>
+      <c r="H66" s="46"/>
+      <c r="I66" s="46"/>
+      <c r="J66" s="46"/>
+      <c r="K66" s="46"/>
+      <c r="L66" s="46"/>
       <c r="M66" s="16"/>
-      <c r="N66" s="16"/>
+      <c r="N66" s="15"/>
       <c r="O66" s="15"/>
       <c r="P66" s="15"/>
       <c r="Q66" s="15"/>
-      <c r="R66" s="12"/>
+      <c r="R66" s="15"/>
     </row>
     <row r="67" spans="4:18" x14ac:dyDescent="0.2">
-      <c r="D67" s="19"/>
-      <c r="E67" s="19"/>
-      <c r="F67" s="19"/>
-      <c r="G67" s="12"/>
-      <c r="H67" s="20"/>
-      <c r="I67" s="12"/>
-      <c r="J67" s="19"/>
-      <c r="K67" s="19"/>
-      <c r="L67" s="19"/>
-      <c r="M67" s="19"/>
-      <c r="N67" s="12"/>
-      <c r="O67" s="20"/>
-      <c r="P67" s="12"/>
-      <c r="Q67" s="19"/>
-      <c r="R67" s="19"/>
+      <c r="D67" s="46"/>
+      <c r="E67" s="46"/>
+      <c r="F67" s="46"/>
+      <c r="G67" s="46"/>
+      <c r="H67" s="46"/>
+      <c r="I67" s="46"/>
+      <c r="J67" s="46"/>
+      <c r="K67" s="46"/>
+      <c r="L67" s="46"/>
+      <c r="M67" s="16"/>
+      <c r="N67" s="15"/>
+      <c r="O67" s="15"/>
+      <c r="P67" s="15"/>
+      <c r="Q67" s="15"/>
+      <c r="R67" s="15"/>
     </row>
     <row r="68" spans="4:18" x14ac:dyDescent="0.2">
-      <c r="D68" s="38"/>
-      <c r="E68" s="12"/>
-      <c r="F68" s="15"/>
-      <c r="G68" s="12"/>
-      <c r="H68" s="12"/>
-      <c r="I68" s="12"/>
-      <c r="J68" s="12"/>
-      <c r="K68" s="12"/>
-      <c r="L68" s="12"/>
+      <c r="D68" s="46"/>
+      <c r="E68" s="46"/>
+      <c r="F68" s="46"/>
+      <c r="G68" s="46"/>
+      <c r="H68" s="46"/>
+      <c r="I68" s="46"/>
+      <c r="J68" s="46"/>
+      <c r="K68" s="46"/>
+      <c r="L68" s="46"/>
       <c r="M68" s="15"/>
-      <c r="N68" s="12"/>
-      <c r="O68" s="12"/>
-      <c r="P68" s="12"/>
-      <c r="Q68" s="12"/>
-      <c r="R68" s="12"/>
+      <c r="N68" s="15"/>
+      <c r="O68" s="16"/>
+      <c r="P68" s="16"/>
+      <c r="Q68" s="15"/>
+      <c r="R68" s="15"/>
     </row>
     <row r="69" spans="4:18" x14ac:dyDescent="0.2">
-      <c r="D69" s="38"/>
-      <c r="E69" s="12"/>
-      <c r="F69" s="12"/>
-      <c r="G69" s="15"/>
-      <c r="H69" s="12"/>
-      <c r="I69" s="12"/>
-      <c r="J69" s="12"/>
-      <c r="K69" s="12"/>
-      <c r="L69" s="12"/>
-      <c r="M69" s="12"/>
+      <c r="D69" s="46"/>
+      <c r="E69" s="46"/>
+      <c r="F69" s="46"/>
+      <c r="G69" s="46"/>
+      <c r="H69" s="46"/>
+      <c r="I69" s="46"/>
+      <c r="J69" s="46"/>
+      <c r="K69" s="46"/>
+      <c r="L69" s="46"/>
+      <c r="M69" s="15"/>
       <c r="N69" s="15"/>
-      <c r="O69" s="12"/>
-      <c r="P69" s="12"/>
-      <c r="Q69" s="12"/>
-      <c r="R69" s="12"/>
+      <c r="O69" s="15"/>
+      <c r="P69" s="15"/>
+      <c r="Q69" s="15"/>
+      <c r="R69" s="15"/>
     </row>
     <row r="70" spans="4:18" x14ac:dyDescent="0.2">
-      <c r="M70" s="39"/>
+      <c r="D70" s="16"/>
+      <c r="E70" s="15"/>
+      <c r="F70" s="15"/>
+      <c r="G70" s="15"/>
+      <c r="H70" s="15"/>
+      <c r="I70" s="15"/>
+      <c r="J70" s="15"/>
+      <c r="K70" s="15"/>
+      <c r="L70" s="15"/>
+      <c r="M70" s="15"/>
+      <c r="N70" s="15"/>
+      <c r="O70" s="15"/>
+      <c r="P70" s="15"/>
+      <c r="Q70" s="15"/>
+      <c r="R70" s="15"/>
+    </row>
+    <row r="71" spans="4:18" x14ac:dyDescent="0.2">
+      <c r="D71" s="33"/>
+      <c r="E71" s="15"/>
+      <c r="F71" s="16"/>
+      <c r="G71" s="16"/>
+      <c r="H71" s="15"/>
+      <c r="I71" s="15"/>
+      <c r="J71" s="15"/>
+      <c r="K71" s="12"/>
+      <c r="L71" s="15"/>
+      <c r="M71" s="16"/>
+      <c r="N71" s="16"/>
+      <c r="O71" s="15"/>
+      <c r="P71" s="15"/>
+      <c r="Q71" s="15"/>
+      <c r="R71" s="12"/>
+    </row>
+    <row r="72" spans="4:18" x14ac:dyDescent="0.2">
+      <c r="D72" s="19"/>
+      <c r="E72" s="19"/>
+      <c r="F72" s="19"/>
+      <c r="G72" s="12"/>
+      <c r="H72" s="20"/>
+      <c r="I72" s="12"/>
+      <c r="J72" s="19"/>
+      <c r="K72" s="19"/>
+      <c r="L72" s="19"/>
+      <c r="M72" s="19"/>
+      <c r="N72" s="12"/>
+      <c r="O72" s="20"/>
+      <c r="P72" s="12"/>
+      <c r="Q72" s="19"/>
+      <c r="R72" s="19"/>
+    </row>
+    <row r="73" spans="4:18" x14ac:dyDescent="0.2">
+      <c r="D73" s="33"/>
+      <c r="E73" s="12"/>
+      <c r="F73" s="15"/>
+      <c r="G73" s="12"/>
+      <c r="H73" s="12"/>
+      <c r="I73" s="12"/>
+      <c r="J73" s="12"/>
+      <c r="K73" s="12"/>
+      <c r="L73" s="12"/>
+      <c r="M73" s="15"/>
+      <c r="N73" s="12"/>
+      <c r="O73" s="12"/>
+      <c r="P73" s="12"/>
+      <c r="Q73" s="12"/>
+      <c r="R73" s="12"/>
+    </row>
+    <row r="74" spans="4:18" x14ac:dyDescent="0.2">
+      <c r="D74" s="33"/>
+      <c r="E74" s="12"/>
+      <c r="F74" s="12"/>
+      <c r="G74" s="15"/>
+      <c r="H74" s="12"/>
+      <c r="I74" s="12"/>
+      <c r="J74" s="12"/>
+      <c r="K74" s="12"/>
+      <c r="L74" s="12"/>
+      <c r="M74" s="12"/>
+      <c r="N74" s="15"/>
+      <c r="O74" s="12"/>
+      <c r="P74" s="12"/>
+      <c r="Q74" s="12"/>
+      <c r="R74" s="12"/>
+    </row>
+    <row r="75" spans="4:18" x14ac:dyDescent="0.2">
+      <c r="M75" s="34"/>
     </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="D55:K55"/>
-    <mergeCell ref="D57:K57"/>
-    <mergeCell ref="A37:C42"/>
-    <mergeCell ref="A44:C45"/>
-    <mergeCell ref="A47:C48"/>
-    <mergeCell ref="A50:C50"/>
-    <mergeCell ref="D53:K53"/>
-    <mergeCell ref="D54:K54"/>
-    <mergeCell ref="A24:C35"/>
+  <mergeCells count="11">
+    <mergeCell ref="D61:L69"/>
+    <mergeCell ref="A29:C40"/>
     <mergeCell ref="D1:K1"/>
-    <mergeCell ref="A5:C22"/>
-    <mergeCell ref="D9:K9"/>
-    <mergeCell ref="D12:K12"/>
-    <mergeCell ref="D19:K19"/>
+    <mergeCell ref="A5:C27"/>
+    <mergeCell ref="D10:K10"/>
+    <mergeCell ref="D24:K24"/>
+    <mergeCell ref="D16:K16"/>
+    <mergeCell ref="A42:C47"/>
+    <mergeCell ref="A49:C50"/>
+    <mergeCell ref="A52:C53"/>
+    <mergeCell ref="A55:C55"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0.3" footer="0.3"/>
-  <pageSetup scale="79" orientation="landscape" verticalDpi="599" r:id="rId1"/>
+  <pageSetup scale="65" orientation="landscape" verticalDpi="599" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added upload and download excel template button
</commit_message>
<xml_diff>
--- a/ScheduleTemplate.xlsx
+++ b/ScheduleTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brian/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{235742D9-F706-6649-85A2-70BF9A543A7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDF9157F-92FC-CD49-802C-35F3F09E0C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9960" yWindow="820" windowWidth="24260" windowHeight="21440" xr2:uid="{FD7B0050-CE21-43C8-88B0-92BFB0830FBD}"/>
+    <workbookView xWindow="9940" yWindow="800" windowWidth="24260" windowHeight="21440" xr2:uid="{FD7B0050-CE21-43C8-88B0-92BFB0830FBD}"/>
   </bookViews>
   <sheets>
     <sheet name="Feb 05- Feb 11" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="59">
   <si>
     <t>Holiday Inn Express Vancouver Airport - Schedule</t>
   </si>
@@ -210,6 +210,9 @@
   </si>
   <si>
     <t>ROBENSON*</t>
+  </si>
+  <si>
+    <t>CARLA</t>
   </si>
 </sst>
 </file>
@@ -548,37 +551,37 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -923,7 +926,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="5.6640625" customWidth="1"/>
@@ -935,29 +938,29 @@
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
     </row>
     <row r="2" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="26"/>
+      <c r="I2" s="26"/>
+      <c r="J2" s="26"/>
+      <c r="K2" s="26"/>
     </row>
     <row r="3" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1"/>
@@ -1024,11 +1027,11 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="26"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="22"/>
       <c r="D5" s="8" t="s">
         <v>10</v>
       </c>
@@ -1041,9 +1044,9 @@
       <c r="K5" s="9"/>
     </row>
     <row r="6" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="27"/>
-      <c r="B6" s="28"/>
-      <c r="C6" s="29"/>
+      <c r="A6" s="28"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="30"/>
       <c r="D6" s="8" t="s">
         <v>12</v>
       </c>
@@ -1056,9 +1059,9 @@
       <c r="K6" s="10"/>
     </row>
     <row r="7" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="27"/>
-      <c r="B7" s="28"/>
-      <c r="C7" s="29"/>
+      <c r="A7" s="28"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="30"/>
       <c r="D7" s="8" t="s">
         <v>13</v>
       </c>
@@ -1071,9 +1074,9 @@
       <c r="K7" s="10"/>
     </row>
     <row r="8" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="27"/>
-      <c r="B8" s="28"/>
-      <c r="C8" s="29"/>
+      <c r="A8" s="28"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="30"/>
       <c r="D8" s="8" t="s">
         <v>14</v>
       </c>
@@ -1086,9 +1089,9 @@
       <c r="K8" s="10"/>
     </row>
     <row r="9" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="27"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="29"/>
+      <c r="A9" s="28"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="30"/>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -1099,22 +1102,22 @@
       <c r="K9" s="10"/>
     </row>
     <row r="10" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="27"/>
-      <c r="B10" s="28"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="23"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="33"/>
+      <c r="I10" s="33"/>
+      <c r="J10" s="33"/>
+      <c r="K10" s="34"/>
     </row>
     <row r="11" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="27"/>
-      <c r="B11" s="28"/>
-      <c r="C11" s="29"/>
+      <c r="A11" s="28"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="30"/>
       <c r="D11" s="8" t="s">
         <v>15</v>
       </c>
@@ -1127,9 +1130,9 @@
       <c r="K11" s="10"/>
     </row>
     <row r="12" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="27"/>
-      <c r="B12" s="28"/>
-      <c r="C12" s="29"/>
+      <c r="A12" s="28"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="30"/>
       <c r="D12" s="8" t="s">
         <v>16</v>
       </c>
@@ -1142,9 +1145,9 @@
       <c r="K12" s="10"/>
     </row>
     <row r="13" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="27"/>
-      <c r="B13" s="28"/>
-      <c r="C13" s="29"/>
+      <c r="A13" s="28"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="30"/>
       <c r="D13" s="8" t="s">
         <v>17</v>
       </c>
@@ -1157,9 +1160,9 @@
       <c r="K13" s="10"/>
     </row>
     <row r="14" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="27"/>
-      <c r="B14" s="28"/>
-      <c r="C14" s="29"/>
+      <c r="A14" s="28"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="30"/>
       <c r="D14" s="8" t="s">
         <v>18</v>
       </c>
@@ -1172,9 +1175,9 @@
       <c r="K14" s="10"/>
     </row>
     <row r="15" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="27"/>
-      <c r="B15" s="28"/>
-      <c r="C15" s="29"/>
+      <c r="A15" s="28"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="30"/>
       <c r="D15" s="8"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
@@ -1185,22 +1188,22 @@
       <c r="K15" s="10"/>
     </row>
     <row r="16" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="27"/>
-      <c r="B16" s="28"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="23"/>
+      <c r="A16" s="28"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="33"/>
+      <c r="K16" s="34"/>
     </row>
     <row r="17" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="27"/>
-      <c r="B17" s="28"/>
-      <c r="C17" s="29"/>
+      <c r="A17" s="28"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="30"/>
       <c r="D17" s="8" t="s">
         <v>19</v>
       </c>
@@ -1213,9 +1216,9 @@
       <c r="K17" s="9"/>
     </row>
     <row r="18" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="27"/>
-      <c r="B18" s="28"/>
-      <c r="C18" s="29"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="30"/>
       <c r="D18" s="8" t="s">
         <v>53</v>
       </c>
@@ -1228,9 +1231,9 @@
       <c r="K18" s="9"/>
     </row>
     <row r="19" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="27"/>
-      <c r="B19" s="28"/>
-      <c r="C19" s="29"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="30"/>
       <c r="D19" s="8" t="s">
         <v>54</v>
       </c>
@@ -1243,9 +1246,9 @@
       <c r="K19" s="10"/>
     </row>
     <row r="20" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="27"/>
-      <c r="B20" s="28"/>
-      <c r="C20" s="29"/>
+      <c r="A20" s="28"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="30"/>
       <c r="D20" s="8" t="s">
         <v>21</v>
       </c>
@@ -1258,9 +1261,9 @@
       <c r="K20" s="10"/>
     </row>
     <row r="21" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="27"/>
-      <c r="B21" s="28"/>
-      <c r="C21" s="29"/>
+      <c r="A21" s="28"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="30"/>
       <c r="D21" s="8" t="s">
         <v>22</v>
       </c>
@@ -1273,9 +1276,9 @@
       <c r="K21" s="10"/>
     </row>
     <row r="22" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="27"/>
-      <c r="B22" s="28"/>
-      <c r="C22" s="29"/>
+      <c r="A22" s="28"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="30"/>
       <c r="D22" s="8"/>
       <c r="E22" s="10"/>
       <c r="F22" s="9"/>
@@ -1286,9 +1289,9 @@
       <c r="K22" s="10"/>
     </row>
     <row r="23" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="27"/>
-      <c r="B23" s="28"/>
-      <c r="C23" s="29"/>
+      <c r="A23" s="28"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="30"/>
       <c r="D23" s="11" t="s">
         <v>23</v>
       </c>
@@ -1301,22 +1304,22 @@
       <c r="K23" s="12"/>
     </row>
     <row r="24" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="27"/>
-      <c r="B24" s="28"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="22"/>
-      <c r="I24" s="22"/>
-      <c r="J24" s="22"/>
-      <c r="K24" s="23"/>
+      <c r="A24" s="28"/>
+      <c r="B24" s="29"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="33"/>
+      <c r="F24" s="33"/>
+      <c r="G24" s="33"/>
+      <c r="H24" s="33"/>
+      <c r="I24" s="33"/>
+      <c r="J24" s="33"/>
+      <c r="K24" s="34"/>
     </row>
     <row r="25" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="27"/>
-      <c r="B25" s="28"/>
-      <c r="C25" s="29"/>
+      <c r="A25" s="28"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="30"/>
       <c r="D25" s="8" t="s">
         <v>24</v>
       </c>
@@ -1343,9 +1346,9 @@
       </c>
     </row>
     <row r="26" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="27"/>
-      <c r="B26" s="28"/>
-      <c r="C26" s="29"/>
+      <c r="A26" s="28"/>
+      <c r="B26" s="29"/>
+      <c r="C26" s="30"/>
       <c r="D26" s="8" t="s">
         <v>25</v>
       </c>
@@ -1372,9 +1375,9 @@
       </c>
     </row>
     <row r="27" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="30"/>
+      <c r="A27" s="23"/>
       <c r="B27" s="31"/>
-      <c r="C27" s="32"/>
+      <c r="C27" s="25"/>
       <c r="D27" s="8" t="s">
         <v>26</v>
       </c>
@@ -1414,11 +1417,11 @@
       <c r="K28" s="5"/>
     </row>
     <row r="29" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="33" t="s">
+      <c r="A29" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="25"/>
-      <c r="C29" s="26"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="22"/>
       <c r="D29" s="10" t="s">
         <v>28</v>
       </c>
@@ -1431,9 +1434,9 @@
       <c r="K29" s="19"/>
     </row>
     <row r="30" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="27"/>
-      <c r="B30" s="28"/>
-      <c r="C30" s="29"/>
+      <c r="A30" s="28"/>
+      <c r="B30" s="29"/>
+      <c r="C30" s="30"/>
       <c r="D30" s="10" t="s">
         <v>29</v>
       </c>
@@ -1446,9 +1449,9 @@
       <c r="K30" s="19"/>
     </row>
     <row r="31" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="27"/>
-      <c r="B31" s="28"/>
-      <c r="C31" s="29"/>
+      <c r="A31" s="28"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="30"/>
       <c r="D31" s="10" t="s">
         <v>30</v>
       </c>
@@ -1461,9 +1464,9 @@
       <c r="K31" s="19"/>
     </row>
     <row r="32" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="27"/>
-      <c r="B32" s="28"/>
-      <c r="C32" s="29"/>
+      <c r="A32" s="28"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="30"/>
       <c r="D32" s="10" t="s">
         <v>31</v>
       </c>
@@ -1476,9 +1479,9 @@
       <c r="K32" s="19"/>
     </row>
     <row r="33" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="27"/>
-      <c r="B33" s="28"/>
-      <c r="C33" s="29"/>
+      <c r="A33" s="28"/>
+      <c r="B33" s="29"/>
+      <c r="C33" s="30"/>
       <c r="D33" s="10" t="s">
         <v>32</v>
       </c>
@@ -1491,9 +1494,9 @@
       <c r="K33" s="19"/>
     </row>
     <row r="34" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="27"/>
-      <c r="B34" s="28"/>
-      <c r="C34" s="29"/>
+      <c r="A34" s="28"/>
+      <c r="B34" s="29"/>
+      <c r="C34" s="30"/>
       <c r="D34" s="10" t="s">
         <v>33</v>
       </c>
@@ -1506,9 +1509,9 @@
       <c r="K34" s="19"/>
     </row>
     <row r="35" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="27"/>
-      <c r="B35" s="28"/>
-      <c r="C35" s="29"/>
+      <c r="A35" s="28"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="30"/>
       <c r="D35" s="10" t="s">
         <v>34</v>
       </c>
@@ -1521,9 +1524,9 @@
       <c r="K35" s="19"/>
     </row>
     <row r="36" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="27"/>
-      <c r="B36" s="28"/>
-      <c r="C36" s="29"/>
+      <c r="A36" s="28"/>
+      <c r="B36" s="29"/>
+      <c r="C36" s="30"/>
       <c r="D36" s="10" t="s">
         <v>57</v>
       </c>
@@ -1536,9 +1539,9 @@
       <c r="K36" s="19"/>
     </row>
     <row r="37" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="27"/>
-      <c r="B37" s="28"/>
-      <c r="C37" s="29"/>
+      <c r="A37" s="28"/>
+      <c r="B37" s="29"/>
+      <c r="C37" s="30"/>
       <c r="D37" s="10" t="s">
         <v>55</v>
       </c>
@@ -1551,9 +1554,9 @@
       <c r="K37" s="19"/>
     </row>
     <row r="38" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="27"/>
-      <c r="B38" s="28"/>
-      <c r="C38" s="29"/>
+      <c r="A38" s="28"/>
+      <c r="B38" s="29"/>
+      <c r="C38" s="30"/>
       <c r="D38" s="10" t="s">
         <v>56</v>
       </c>
@@ -1566,9 +1569,9 @@
       <c r="K38" s="19"/>
     </row>
     <row r="39" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="27"/>
-      <c r="B39" s="28"/>
-      <c r="C39" s="29"/>
+      <c r="A39" s="28"/>
+      <c r="B39" s="29"/>
+      <c r="C39" s="30"/>
       <c r="D39" s="10"/>
       <c r="E39" s="19"/>
       <c r="F39" s="19"/>
@@ -1579,9 +1582,9 @@
       <c r="K39" s="19"/>
     </row>
     <row r="40" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="27"/>
-      <c r="B40" s="28"/>
-      <c r="C40" s="29"/>
+      <c r="A40" s="28"/>
+      <c r="B40" s="29"/>
+      <c r="C40" s="30"/>
       <c r="D40" s="13" t="s">
         <v>35</v>
       </c>
@@ -1594,9 +1597,9 @@
       <c r="K40" s="13"/>
     </row>
     <row r="41" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="30"/>
-      <c r="B41" s="34"/>
-      <c r="C41" s="32"/>
+      <c r="A41" s="23"/>
+      <c r="B41" s="24"/>
+      <c r="C41" s="25"/>
       <c r="D41" s="3" t="s">
         <v>36</v>
       </c>
@@ -1622,11 +1625,11 @@
       <c r="K42" s="14"/>
     </row>
     <row r="43" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="33" t="s">
+      <c r="A43" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="B43" s="25"/>
-      <c r="C43" s="26"/>
+      <c r="B43" s="21"/>
+      <c r="C43" s="22"/>
       <c r="D43" s="10" t="s">
         <v>38</v>
       </c>
@@ -1639,9 +1642,9 @@
       <c r="K43" s="10"/>
     </row>
     <row r="44" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="27"/>
-      <c r="B44" s="28"/>
-      <c r="C44" s="29"/>
+      <c r="A44" s="28"/>
+      <c r="B44" s="29"/>
+      <c r="C44" s="30"/>
       <c r="D44" s="10" t="s">
         <v>39</v>
       </c>
@@ -1654,9 +1657,9 @@
       <c r="K44" s="10"/>
     </row>
     <row r="45" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="27"/>
-      <c r="B45" s="28"/>
-      <c r="C45" s="29"/>
+      <c r="A45" s="28"/>
+      <c r="B45" s="29"/>
+      <c r="C45" s="30"/>
       <c r="D45" s="10" t="s">
         <v>40</v>
       </c>
@@ -1669,9 +1672,9 @@
       <c r="K45" s="17"/>
     </row>
     <row r="46" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="27"/>
-      <c r="B46" s="28"/>
-      <c r="C46" s="29"/>
+      <c r="A46" s="28"/>
+      <c r="B46" s="29"/>
+      <c r="C46" s="30"/>
       <c r="D46" s="10" t="s">
         <v>41</v>
       </c>
@@ -1684,9 +1687,9 @@
       <c r="K46" s="10"/>
     </row>
     <row r="47" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="27"/>
-      <c r="B47" s="28"/>
-      <c r="C47" s="29"/>
+      <c r="A47" s="28"/>
+      <c r="B47" s="29"/>
+      <c r="C47" s="30"/>
       <c r="D47" s="10" t="s">
         <v>42</v>
       </c>
@@ -1699,188 +1702,216 @@
       <c r="K47" s="10"/>
     </row>
     <row r="48" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="30"/>
-      <c r="B48" s="34"/>
-      <c r="C48" s="32"/>
+      <c r="A48" s="28"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="30"/>
       <c r="D48" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="E48" s="10"/>
+      <c r="E48" s="17"/>
       <c r="F48" s="10"/>
       <c r="G48" s="10"/>
       <c r="H48" s="10"/>
       <c r="I48" s="10"/>
-      <c r="J48" s="10"/>
+      <c r="J48" s="17"/>
       <c r="K48" s="10"/>
     </row>
     <row r="49" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="1"/>
-      <c r="B49" s="1"/>
-      <c r="C49" s="1"/>
-      <c r="D49" s="5"/>
-      <c r="E49" s="5"/>
-      <c r="F49" s="5"/>
-      <c r="G49" s="5"/>
-      <c r="H49" s="5"/>
-      <c r="I49" s="5"/>
-      <c r="J49" s="5"/>
-      <c r="K49" s="5"/>
+      <c r="A49" s="28"/>
+      <c r="B49" s="29"/>
+      <c r="C49" s="30"/>
+      <c r="D49" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E49" s="17"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+      <c r="I49" s="10"/>
+      <c r="J49" s="17"/>
+      <c r="K49" s="10"/>
     </row>
     <row r="50" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="35" t="s">
+      <c r="A50" s="23"/>
+      <c r="B50" s="24"/>
+      <c r="C50" s="25"/>
+      <c r="D50" s="10"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="10"/>
+      <c r="H50" s="10"/>
+      <c r="I50" s="10"/>
+      <c r="J50" s="10"/>
+      <c r="K50" s="10"/>
+    </row>
+    <row r="51" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="1"/>
+      <c r="B51" s="1"/>
+      <c r="C51" s="1"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="K51" s="5"/>
+    </row>
+    <row r="52" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="B50" s="25"/>
-      <c r="C50" s="26"/>
-      <c r="D50" s="17" t="s">
+      <c r="B52" s="21"/>
+      <c r="C52" s="22"/>
+      <c r="D52" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E50" s="10" t="s">
+      <c r="E52" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="F50" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="G50" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="H50" s="10" t="s">
+      <c r="F52" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="G52" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="H52" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="I50" s="10" t="s">
+      <c r="I52" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="J50" s="10" t="s">
+      <c r="J52" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="K50" s="10" t="s">
+      <c r="K52" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="36"/>
-      <c r="B51" s="37"/>
-      <c r="C51" s="29"/>
-      <c r="D51" s="17" t="s">
+    <row r="53" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="36"/>
+      <c r="B53" s="37"/>
+      <c r="C53" s="30"/>
+      <c r="D53" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="E51" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="F51" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="G51" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="H51" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="I51" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="J51" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="K51" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="30"/>
-      <c r="B52" s="34"/>
-      <c r="C52" s="32"/>
-      <c r="D52" s="17"/>
-      <c r="E52" s="18"/>
-      <c r="F52" s="18"/>
-      <c r="G52" s="18"/>
-      <c r="H52" s="18"/>
-      <c r="I52" s="18"/>
-      <c r="J52" s="18"/>
-      <c r="K52" s="10"/>
-    </row>
-    <row r="53" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="1"/>
-      <c r="B53" s="1"/>
-      <c r="C53" s="1"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="14"/>
-      <c r="F53" s="14"/>
-      <c r="G53" s="5"/>
-      <c r="H53" s="14"/>
-      <c r="I53" s="14"/>
-      <c r="J53" s="14"/>
-      <c r="K53" s="14"/>
+      <c r="E53" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="F53" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="G53" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="H53" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="I53" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="J53" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="K53" s="10" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="54" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="33" t="s">
+      <c r="A54" s="23"/>
+      <c r="B54" s="24"/>
+      <c r="C54" s="25"/>
+      <c r="D54" s="17"/>
+      <c r="E54" s="18"/>
+      <c r="F54" s="18"/>
+      <c r="G54" s="18"/>
+      <c r="H54" s="18"/>
+      <c r="I54" s="18"/>
+      <c r="J54" s="18"/>
+      <c r="K54" s="10"/>
+    </row>
+    <row r="55" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="1"/>
+      <c r="B55" s="1"/>
+      <c r="C55" s="1"/>
+      <c r="D55" s="14"/>
+      <c r="E55" s="14"/>
+      <c r="F55" s="14"/>
+      <c r="G55" s="5"/>
+      <c r="H55" s="14"/>
+      <c r="I55" s="14"/>
+      <c r="J55" s="14"/>
+      <c r="K55" s="14"/>
+    </row>
+    <row r="56" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="B54" s="25"/>
-      <c r="C54" s="26"/>
-      <c r="D54" s="8" t="s">
+      <c r="B56" s="21"/>
+      <c r="C56" s="22"/>
+      <c r="D56" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="E54" s="10" t="s">
+      <c r="E56" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="F54" s="10" t="s">
+      <c r="F56" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="G54" s="10" t="s">
+      <c r="G56" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H54" s="10" t="s">
+      <c r="H56" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="I54" s="10" t="s">
+      <c r="I56" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="J54" s="10" t="s">
+      <c r="J56" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="K54" s="10" t="s">
+      <c r="K56" s="10" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="30"/>
-      <c r="B55" s="34"/>
-      <c r="C55" s="32"/>
-      <c r="D55" s="17" t="s">
+    <row r="57" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="23"/>
+      <c r="B57" s="24"/>
+      <c r="C57" s="25"/>
+      <c r="D57" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="E55" s="10" t="s">
+      <c r="E57" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="F55" s="10" t="s">
+      <c r="F57" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="G55" s="10" t="s">
+      <c r="G57" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H55" s="9" t="s">
+      <c r="H57" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="I55" s="9" t="s">
+      <c r="I57" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="J55" s="9" t="s">
+      <c r="J57" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="K55" s="9" t="s">
+      <c r="K57" s="9" t="s">
         <v>51</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A54:C55"/>
+    <mergeCell ref="A56:C57"/>
     <mergeCell ref="D1:K2"/>
     <mergeCell ref="A5:C27"/>
     <mergeCell ref="D24:K24"/>
     <mergeCell ref="A29:C41"/>
-    <mergeCell ref="A43:C48"/>
-    <mergeCell ref="A50:C52"/>
+    <mergeCell ref="A43:C50"/>
+    <mergeCell ref="A52:C54"/>
     <mergeCell ref="D10:K10"/>
     <mergeCell ref="D16:K16"/>
   </mergeCells>

</xml_diff>

<commit_message>
fixed bugs and updated color scheming
</commit_message>
<xml_diff>
--- a/ScheduleTemplate.xlsx
+++ b/ScheduleTemplate.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brian/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDF9157F-92FC-CD49-802C-35F3F09E0C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACF09C29-BC5B-F249-9EF0-87FCD773725C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9940" yWindow="800" windowWidth="24260" windowHeight="21440" xr2:uid="{FD7B0050-CE21-43C8-88B0-92BFB0830FBD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="60">
   <si>
     <t>Holiday Inn Express Vancouver Airport - Schedule</t>
   </si>
@@ -113,12 +113,6 @@
     <t>IAN</t>
   </si>
   <si>
-    <t>SARA</t>
-  </si>
-  <si>
-    <t>JORDAN</t>
-  </si>
-  <si>
     <t>Shuttle Drivers</t>
   </si>
   <si>
@@ -213,6 +207,15 @@
   </si>
   <si>
     <t>CARLA</t>
+  </si>
+  <si>
+    <t>SAMUEL</t>
+  </si>
+  <si>
+    <t>JAKRA</t>
+  </si>
+  <si>
+    <t>RONALD</t>
   </si>
 </sst>
 </file>
@@ -346,7 +349,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -379,19 +382,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -492,7 +482,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -515,7 +505,7 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -524,7 +514,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -554,41 +544,42 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -926,7 +917,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K57"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="5.6640625" customWidth="1"/>
@@ -967,7 +958,7 @@
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E3" s="6">
         <v>46058</v>
@@ -1027,11 +1018,11 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="27" t="s">
+      <c r="A5" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="21"/>
-      <c r="C5" s="22"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
       <c r="D5" s="8" t="s">
         <v>10</v>
       </c>
@@ -1044,9 +1035,9 @@
       <c r="K5" s="9"/>
     </row>
     <row r="6" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="28"/>
-      <c r="B6" s="29"/>
-      <c r="C6" s="30"/>
+      <c r="A6" s="37"/>
+      <c r="B6" s="38"/>
+      <c r="C6" s="37"/>
       <c r="D6" s="8" t="s">
         <v>12</v>
       </c>
@@ -1059,9 +1050,9 @@
       <c r="K6" s="10"/>
     </row>
     <row r="7" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="28"/>
-      <c r="B7" s="29"/>
-      <c r="C7" s="30"/>
+      <c r="A7" s="37"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="37"/>
       <c r="D7" s="8" t="s">
         <v>13</v>
       </c>
@@ -1074,9 +1065,9 @@
       <c r="K7" s="10"/>
     </row>
     <row r="8" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="28"/>
-      <c r="B8" s="29"/>
-      <c r="C8" s="30"/>
+      <c r="A8" s="37"/>
+      <c r="B8" s="38"/>
+      <c r="C8" s="37"/>
       <c r="D8" s="8" t="s">
         <v>14</v>
       </c>
@@ -1089,9 +1080,9 @@
       <c r="K8" s="10"/>
     </row>
     <row r="9" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="28"/>
-      <c r="B9" s="29"/>
-      <c r="C9" s="30"/>
+      <c r="A9" s="37"/>
+      <c r="B9" s="38"/>
+      <c r="C9" s="37"/>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -1102,22 +1093,22 @@
       <c r="K9" s="10"/>
     </row>
     <row r="10" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="28"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="33"/>
-      <c r="G10" s="33"/>
-      <c r="H10" s="33"/>
-      <c r="I10" s="33"/>
-      <c r="J10" s="33"/>
-      <c r="K10" s="34"/>
+      <c r="A10" s="37"/>
+      <c r="B10" s="38"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="31"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="32"/>
     </row>
     <row r="11" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="28"/>
-      <c r="B11" s="29"/>
-      <c r="C11" s="30"/>
+      <c r="A11" s="37"/>
+      <c r="B11" s="38"/>
+      <c r="C11" s="37"/>
       <c r="D11" s="8" t="s">
         <v>15</v>
       </c>
@@ -1130,9 +1121,9 @@
       <c r="K11" s="10"/>
     </row>
     <row r="12" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="28"/>
-      <c r="B12" s="29"/>
-      <c r="C12" s="30"/>
+      <c r="A12" s="37"/>
+      <c r="B12" s="38"/>
+      <c r="C12" s="37"/>
       <c r="D12" s="8" t="s">
         <v>16</v>
       </c>
@@ -1145,9 +1136,9 @@
       <c r="K12" s="10"/>
     </row>
     <row r="13" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="28"/>
-      <c r="B13" s="29"/>
-      <c r="C13" s="30"/>
+      <c r="A13" s="37"/>
+      <c r="B13" s="38"/>
+      <c r="C13" s="37"/>
       <c r="D13" s="8" t="s">
         <v>17</v>
       </c>
@@ -1160,9 +1151,9 @@
       <c r="K13" s="10"/>
     </row>
     <row r="14" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="28"/>
-      <c r="B14" s="29"/>
-      <c r="C14" s="30"/>
+      <c r="A14" s="37"/>
+      <c r="B14" s="38"/>
+      <c r="C14" s="37"/>
       <c r="D14" s="8" t="s">
         <v>18</v>
       </c>
@@ -1175,9 +1166,9 @@
       <c r="K14" s="10"/>
     </row>
     <row r="15" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="28"/>
-      <c r="B15" s="29"/>
-      <c r="C15" s="30"/>
+      <c r="A15" s="37"/>
+      <c r="B15" s="38"/>
+      <c r="C15" s="37"/>
       <c r="D15" s="8"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
@@ -1188,22 +1179,22 @@
       <c r="K15" s="10"/>
     </row>
     <row r="16" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="28"/>
-      <c r="B16" s="29"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="33"/>
-      <c r="H16" s="33"/>
-      <c r="I16" s="33"/>
-      <c r="J16" s="33"/>
-      <c r="K16" s="34"/>
+      <c r="A16" s="37"/>
+      <c r="B16" s="38"/>
+      <c r="C16" s="37"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+      <c r="I16" s="31"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="32"/>
     </row>
     <row r="17" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="28"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="30"/>
+      <c r="A17" s="37"/>
+      <c r="B17" s="38"/>
+      <c r="C17" s="37"/>
       <c r="D17" s="8" t="s">
         <v>19</v>
       </c>
@@ -1216,11 +1207,11 @@
       <c r="K17" s="9"/>
     </row>
     <row r="18" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="28"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="30"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="38"/>
+      <c r="C18" s="37"/>
       <c r="D18" s="8" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="10"/>
@@ -1231,11 +1222,11 @@
       <c r="K18" s="9"/>
     </row>
     <row r="19" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="28"/>
-      <c r="B19" s="29"/>
-      <c r="C19" s="30"/>
+      <c r="A19" s="37"/>
+      <c r="B19" s="38"/>
+      <c r="C19" s="37"/>
       <c r="D19" s="8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
@@ -1246,9 +1237,9 @@
       <c r="K19" s="10"/>
     </row>
     <row r="20" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="28"/>
-      <c r="B20" s="29"/>
-      <c r="C20" s="30"/>
+      <c r="A20" s="37"/>
+      <c r="B20" s="38"/>
+      <c r="C20" s="37"/>
       <c r="D20" s="8" t="s">
         <v>21</v>
       </c>
@@ -1261,9 +1252,9 @@
       <c r="K20" s="10"/>
     </row>
     <row r="21" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="28"/>
-      <c r="B21" s="29"/>
-      <c r="C21" s="30"/>
+      <c r="A21" s="37"/>
+      <c r="B21" s="38"/>
+      <c r="C21" s="37"/>
       <c r="D21" s="8" t="s">
         <v>22</v>
       </c>
@@ -1276,9 +1267,9 @@
       <c r="K21" s="10"/>
     </row>
     <row r="22" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="28"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="30"/>
+      <c r="A22" s="37"/>
+      <c r="B22" s="38"/>
+      <c r="C22" s="37"/>
       <c r="D22" s="8"/>
       <c r="E22" s="10"/>
       <c r="F22" s="9"/>
@@ -1289,9 +1280,9 @@
       <c r="K22" s="10"/>
     </row>
     <row r="23" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="28"/>
-      <c r="B23" s="29"/>
-      <c r="C23" s="30"/>
+      <c r="A23" s="37"/>
+      <c r="B23" s="38"/>
+      <c r="C23" s="37"/>
       <c r="D23" s="11" t="s">
         <v>23</v>
       </c>
@@ -1304,22 +1295,22 @@
       <c r="K23" s="12"/>
     </row>
     <row r="24" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="28"/>
-      <c r="B24" s="29"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="33"/>
-      <c r="G24" s="33"/>
-      <c r="H24" s="33"/>
-      <c r="I24" s="33"/>
-      <c r="J24" s="33"/>
-      <c r="K24" s="34"/>
+      <c r="A24" s="37"/>
+      <c r="B24" s="38"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="31"/>
+      <c r="F24" s="31"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="31"/>
+      <c r="J24" s="31"/>
+      <c r="K24" s="32"/>
     </row>
     <row r="25" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="28"/>
-      <c r="B25" s="29"/>
-      <c r="C25" s="30"/>
+      <c r="A25" s="37"/>
+      <c r="B25" s="38"/>
+      <c r="C25" s="37"/>
       <c r="D25" s="8" t="s">
         <v>24</v>
       </c>
@@ -1346,82 +1337,54 @@
       </c>
     </row>
     <row r="26" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="28"/>
-      <c r="B26" s="29"/>
-      <c r="C26" s="30"/>
-      <c r="D26" s="8" t="s">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+      <c r="C26" s="1"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+    </row>
+    <row r="27" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="E26" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F26" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G26" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="H26" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="I26" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="J26" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="K26" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="23"/>
-      <c r="B27" s="31"/>
-      <c r="C27" s="25"/>
-      <c r="D27" s="8" t="s">
+      <c r="B27" s="21"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="E27" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F27" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G27" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="H27" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="I27" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="J27" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="K27" s="10" t="s">
-        <v>11</v>
-      </c>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
+      <c r="G27" s="19"/>
+      <c r="H27" s="19"/>
+      <c r="I27" s="19"/>
+      <c r="J27" s="19"/>
+      <c r="K27" s="19"/>
     </row>
     <row r="28" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
+      <c r="A28" s="27"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="19"/>
+      <c r="H28" s="19"/>
+      <c r="I28" s="19"/>
+      <c r="J28" s="19"/>
+      <c r="K28" s="19"/>
     </row>
     <row r="29" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="B29" s="21"/>
-      <c r="C29" s="22"/>
+      <c r="A29" s="27"/>
+      <c r="B29" s="28"/>
+      <c r="C29" s="29"/>
       <c r="D29" s="10" t="s">
         <v>28</v>
       </c>
@@ -1434,9 +1397,9 @@
       <c r="K29" s="19"/>
     </row>
     <row r="30" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="28"/>
-      <c r="B30" s="29"/>
-      <c r="C30" s="30"/>
+      <c r="A30" s="27"/>
+      <c r="B30" s="28"/>
+      <c r="C30" s="29"/>
       <c r="D30" s="10" t="s">
         <v>29</v>
       </c>
@@ -1449,9 +1412,9 @@
       <c r="K30" s="19"/>
     </row>
     <row r="31" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="28"/>
-      <c r="B31" s="29"/>
-      <c r="C31" s="30"/>
+      <c r="A31" s="27"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="29"/>
       <c r="D31" s="10" t="s">
         <v>30</v>
       </c>
@@ -1464,9 +1427,9 @@
       <c r="K31" s="19"/>
     </row>
     <row r="32" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="28"/>
-      <c r="B32" s="29"/>
-      <c r="C32" s="30"/>
+      <c r="A32" s="27"/>
+      <c r="B32" s="28"/>
+      <c r="C32" s="29"/>
       <c r="D32" s="10" t="s">
         <v>31</v>
       </c>
@@ -1479,9 +1442,9 @@
       <c r="K32" s="19"/>
     </row>
     <row r="33" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="28"/>
-      <c r="B33" s="29"/>
-      <c r="C33" s="30"/>
+      <c r="A33" s="27"/>
+      <c r="B33" s="28"/>
+      <c r="C33" s="29"/>
       <c r="D33" s="10" t="s">
         <v>32</v>
       </c>
@@ -1494,11 +1457,11 @@
       <c r="K33" s="19"/>
     </row>
     <row r="34" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="28"/>
-      <c r="B34" s="29"/>
-      <c r="C34" s="30"/>
+      <c r="A34" s="27"/>
+      <c r="B34" s="28"/>
+      <c r="C34" s="29"/>
       <c r="D34" s="10" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
       <c r="E34" s="19"/>
       <c r="F34" s="19"/>
@@ -1509,11 +1472,11 @@
       <c r="K34" s="19"/>
     </row>
     <row r="35" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="28"/>
-      <c r="B35" s="29"/>
-      <c r="C35" s="30"/>
+      <c r="A35" s="27"/>
+      <c r="B35" s="28"/>
+      <c r="C35" s="29"/>
       <c r="D35" s="10" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="E35" s="19"/>
       <c r="F35" s="19"/>
@@ -1524,11 +1487,11 @@
       <c r="K35" s="19"/>
     </row>
     <row r="36" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="28"/>
-      <c r="B36" s="29"/>
-      <c r="C36" s="30"/>
+      <c r="A36" s="27"/>
+      <c r="B36" s="28"/>
+      <c r="C36" s="29"/>
       <c r="D36" s="10" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E36" s="19"/>
       <c r="F36" s="19"/>
@@ -1539,11 +1502,11 @@
       <c r="K36" s="19"/>
     </row>
     <row r="37" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="28"/>
-      <c r="B37" s="29"/>
-      <c r="C37" s="30"/>
+      <c r="A37" s="27"/>
+      <c r="B37" s="28"/>
+      <c r="C37" s="29"/>
       <c r="D37" s="10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E37" s="19"/>
       <c r="F37" s="19"/>
@@ -1554,11 +1517,11 @@
       <c r="K37" s="19"/>
     </row>
     <row r="38" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="28"/>
-      <c r="B38" s="29"/>
-      <c r="C38" s="30"/>
+      <c r="A38" s="27"/>
+      <c r="B38" s="28"/>
+      <c r="C38" s="29"/>
       <c r="D38" s="10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E38" s="19"/>
       <c r="F38" s="19"/>
@@ -1569,10 +1532,12 @@
       <c r="K38" s="19"/>
     </row>
     <row r="39" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="28"/>
-      <c r="B39" s="29"/>
-      <c r="C39" s="30"/>
-      <c r="D39" s="10"/>
+      <c r="A39" s="27"/>
+      <c r="B39" s="28"/>
+      <c r="C39" s="29"/>
+      <c r="D39" s="10" t="s">
+        <v>59</v>
+      </c>
       <c r="E39" s="19"/>
       <c r="F39" s="19"/>
       <c r="G39" s="19"/>
@@ -1582,131 +1547,129 @@
       <c r="K39" s="19"/>
     </row>
     <row r="40" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="28"/>
-      <c r="B40" s="29"/>
-      <c r="C40" s="30"/>
-      <c r="D40" s="13" t="s">
+      <c r="A40" s="27"/>
+      <c r="B40" s="28"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="19"/>
+      <c r="H40" s="19"/>
+      <c r="I40" s="19"/>
+      <c r="J40" s="19"/>
+      <c r="K40" s="19"/>
+    </row>
+    <row r="41" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="27"/>
+      <c r="B41" s="28"/>
+      <c r="C41" s="29"/>
+      <c r="D41" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="E41" s="13"/>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="13"/>
+      <c r="I41" s="13"/>
+      <c r="J41" s="13"/>
+      <c r="K41" s="13"/>
+    </row>
+    <row r="42" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="23"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="3"/>
+    </row>
+    <row r="43" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="1"/>
+      <c r="B43" s="1"/>
+      <c r="C43" s="1"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+      <c r="G43" s="14"/>
+      <c r="H43" s="15"/>
+      <c r="I43" s="14"/>
+      <c r="J43" s="14"/>
+      <c r="K43" s="14"/>
+    </row>
+    <row r="44" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="E40" s="13"/>
-      <c r="F40" s="13"/>
-      <c r="G40" s="13"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="13"/>
-      <c r="J40" s="13"/>
-      <c r="K40" s="13"/>
-    </row>
-    <row r="41" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="23"/>
-      <c r="B41" s="24"/>
-      <c r="C41" s="25"/>
-      <c r="D41" s="3" t="s">
+      <c r="B44" s="21"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-      <c r="G41" s="3"/>
-      <c r="H41" s="3"/>
-      <c r="I41" s="3"/>
-      <c r="J41" s="3"/>
-      <c r="K41" s="3"/>
-    </row>
-    <row r="42" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="1"/>
-      <c r="B42" s="1"/>
-      <c r="C42" s="1"/>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="14"/>
-      <c r="G42" s="14"/>
-      <c r="H42" s="15"/>
-      <c r="I42" s="14"/>
-      <c r="J42" s="14"/>
-      <c r="K42" s="14"/>
-    </row>
-    <row r="43" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="20" t="s">
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="16"/>
+      <c r="I44" s="16"/>
+      <c r="J44" s="10"/>
+      <c r="K44" s="10"/>
+    </row>
+    <row r="45" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="27"/>
+      <c r="B45" s="28"/>
+      <c r="C45" s="29"/>
+      <c r="D45" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B43" s="21"/>
-      <c r="C43" s="22"/>
-      <c r="D43" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="E43" s="10"/>
-      <c r="F43" s="10"/>
-      <c r="G43" s="10"/>
-      <c r="H43" s="16"/>
-      <c r="I43" s="16"/>
-      <c r="J43" s="10"/>
-      <c r="K43" s="10"/>
-    </row>
-    <row r="44" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="28"/>
-      <c r="B44" s="29"/>
-      <c r="C44" s="30"/>
-      <c r="D44" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="E44" s="10"/>
-      <c r="F44" s="17"/>
-      <c r="G44" s="17"/>
-      <c r="H44" s="10"/>
-      <c r="I44" s="10"/>
-      <c r="J44" s="17"/>
-      <c r="K44" s="10"/>
-    </row>
-    <row r="45" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="28"/>
-      <c r="B45" s="29"/>
-      <c r="C45" s="30"/>
-      <c r="D45" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E45" s="17"/>
-      <c r="F45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="17"/>
       <c r="G45" s="17"/>
-      <c r="H45" s="17"/>
+      <c r="H45" s="10"/>
       <c r="I45" s="10"/>
       <c r="J45" s="17"/>
-      <c r="K45" s="17"/>
+      <c r="K45" s="10"/>
     </row>
     <row r="46" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="28"/>
-      <c r="B46" s="29"/>
-      <c r="C46" s="30"/>
+      <c r="A46" s="27"/>
+      <c r="B46" s="28"/>
+      <c r="C46" s="29"/>
       <c r="D46" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="E46" s="10"/>
+        <v>38</v>
+      </c>
+      <c r="E46" s="17"/>
       <c r="F46" s="10"/>
       <c r="G46" s="17"/>
       <c r="H46" s="17"/>
       <c r="I46" s="10"/>
-      <c r="J46" s="10"/>
-      <c r="K46" s="10"/>
+      <c r="J46" s="17"/>
+      <c r="K46" s="17"/>
     </row>
     <row r="47" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="28"/>
-      <c r="B47" s="29"/>
-      <c r="C47" s="30"/>
+      <c r="A47" s="27"/>
+      <c r="B47" s="28"/>
+      <c r="C47" s="29"/>
       <c r="D47" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="E47" s="17"/>
+        <v>39</v>
+      </c>
+      <c r="E47" s="10"/>
       <c r="F47" s="10"/>
-      <c r="G47" s="10"/>
-      <c r="H47" s="10"/>
+      <c r="G47" s="17"/>
+      <c r="H47" s="17"/>
       <c r="I47" s="10"/>
-      <c r="J47" s="17"/>
+      <c r="J47" s="10"/>
       <c r="K47" s="10"/>
     </row>
     <row r="48" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="28"/>
-      <c r="B48" s="29"/>
-      <c r="C48" s="30"/>
+      <c r="A48" s="27"/>
+      <c r="B48" s="28"/>
+      <c r="C48" s="29"/>
       <c r="D48" s="10" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E48" s="17"/>
       <c r="F48" s="10"/>
@@ -1717,11 +1680,11 @@
       <c r="K48" s="10"/>
     </row>
     <row r="49" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="28"/>
-      <c r="B49" s="29"/>
-      <c r="C49" s="30"/>
+      <c r="A49" s="27"/>
+      <c r="B49" s="28"/>
+      <c r="C49" s="29"/>
       <c r="D49" s="10" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="E49" s="17"/>
       <c r="F49" s="10"/>
@@ -1732,186 +1695,201 @@
       <c r="K49" s="10"/>
     </row>
     <row r="50" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="23"/>
-      <c r="B50" s="24"/>
-      <c r="C50" s="25"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="10"/>
+      <c r="A50" s="27"/>
+      <c r="B50" s="28"/>
+      <c r="C50" s="29"/>
+      <c r="D50" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="E50" s="17"/>
       <c r="F50" s="10"/>
       <c r="G50" s="10"/>
       <c r="H50" s="10"/>
       <c r="I50" s="10"/>
-      <c r="J50" s="10"/>
+      <c r="J50" s="17"/>
       <c r="K50" s="10"/>
     </row>
     <row r="51" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="1"/>
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
-      <c r="G51" s="5"/>
-      <c r="H51" s="5"/>
-      <c r="I51" s="5"/>
-      <c r="J51" s="5"/>
-      <c r="K51" s="5"/>
+      <c r="A51" s="23"/>
+      <c r="B51" s="24"/>
+      <c r="C51" s="25"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="10"/>
+      <c r="H51" s="10"/>
+      <c r="I51" s="10"/>
+      <c r="J51" s="10"/>
+      <c r="K51" s="10"/>
     </row>
     <row r="52" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="35" t="s">
+      <c r="A52" s="1"/>
+      <c r="B52" s="1"/>
+      <c r="C52" s="1"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5"/>
+      <c r="I52" s="5"/>
+      <c r="J52" s="5"/>
+      <c r="K52" s="5"/>
+    </row>
+    <row r="53" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="33" t="s">
+        <v>42</v>
+      </c>
+      <c r="B53" s="21"/>
+      <c r="C53" s="22"/>
+      <c r="D53" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="E53" s="10" t="s">
         <v>44</v>
-      </c>
-      <c r="B52" s="21"/>
-      <c r="C52" s="22"/>
-      <c r="D52" s="17" t="s">
-        <v>45</v>
-      </c>
-      <c r="E52" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="F52" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="G52" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="H52" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="I52" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="J52" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="K52" s="10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="36"/>
-      <c r="B53" s="37"/>
-      <c r="C53" s="30"/>
-      <c r="D53" s="17" t="s">
-        <v>47</v>
-      </c>
-      <c r="E53" s="18" t="s">
-        <v>11</v>
       </c>
       <c r="F53" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="G53" s="18" t="s">
+      <c r="G53" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H53" s="18" t="s">
+      <c r="H53" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="I53" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="J53" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="K53" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="34"/>
+      <c r="B54" s="35"/>
+      <c r="C54" s="29"/>
+      <c r="D54" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="E54" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="I53" s="18" t="s">
+      <c r="F54" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="J53" s="18" t="s">
+      <c r="G54" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="K53" s="10" t="s">
+      <c r="H54" s="18" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="54" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="23"/>
-      <c r="B54" s="24"/>
-      <c r="C54" s="25"/>
-      <c r="D54" s="17"/>
-      <c r="E54" s="18"/>
-      <c r="F54" s="18"/>
-      <c r="G54" s="18"/>
-      <c r="H54" s="18"/>
-      <c r="I54" s="18"/>
-      <c r="J54" s="18"/>
-      <c r="K54" s="10"/>
+      <c r="I54" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="J54" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="K54" s="10" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="55" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="1"/>
-      <c r="B55" s="1"/>
-      <c r="C55" s="1"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
-      <c r="F55" s="14"/>
-      <c r="G55" s="5"/>
-      <c r="H55" s="14"/>
-      <c r="I55" s="14"/>
-      <c r="J55" s="14"/>
-      <c r="K55" s="14"/>
+      <c r="A55" s="23"/>
+      <c r="B55" s="24"/>
+      <c r="C55" s="25"/>
+      <c r="D55" s="17"/>
+      <c r="E55" s="18"/>
+      <c r="F55" s="18"/>
+      <c r="G55" s="18"/>
+      <c r="H55" s="18"/>
+      <c r="I55" s="18"/>
+      <c r="J55" s="18"/>
+      <c r="K55" s="10"/>
     </row>
     <row r="56" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="20" t="s">
-        <v>48</v>
-      </c>
-      <c r="B56" s="21"/>
-      <c r="C56" s="22"/>
-      <c r="D56" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="E56" s="10" t="s">
+      <c r="A56" s="1"/>
+      <c r="B56" s="1"/>
+      <c r="C56" s="1"/>
+      <c r="D56" s="14"/>
+      <c r="E56" s="14"/>
+      <c r="F56" s="14"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="14"/>
+      <c r="I56" s="14"/>
+      <c r="J56" s="14"/>
+      <c r="K56" s="14"/>
+    </row>
+    <row r="57" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="F56" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="G56" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="H56" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="I56" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="J56" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="K56" s="10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="23"/>
-      <c r="B57" s="24"/>
-      <c r="C57" s="25"/>
-      <c r="D57" s="17" t="s">
-        <v>50</v>
+      <c r="B57" s="21"/>
+      <c r="C57" s="22"/>
+      <c r="D57" s="8" t="s">
+        <v>47</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="F57" s="10" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="G57" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H57" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="I57" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="J57" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="K57" s="9" t="s">
-        <v>51</v>
+      <c r="H57" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="I57" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="J57" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="K57" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="23"/>
+      <c r="B58" s="24"/>
+      <c r="C58" s="25"/>
+      <c r="D58" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="E58" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F58" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="G58" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="H58" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="I58" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="J58" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="K58" s="9" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A56:C57"/>
+    <mergeCell ref="A57:C58"/>
     <mergeCell ref="D1:K2"/>
-    <mergeCell ref="A5:C27"/>
+    <mergeCell ref="A5:C25"/>
     <mergeCell ref="D24:K24"/>
-    <mergeCell ref="A29:C41"/>
-    <mergeCell ref="A43:C50"/>
-    <mergeCell ref="A52:C54"/>
+    <mergeCell ref="A27:C42"/>
+    <mergeCell ref="A44:C51"/>
+    <mergeCell ref="A53:C55"/>
     <mergeCell ref="D10:K10"/>
     <mergeCell ref="D16:K16"/>
   </mergeCells>

</xml_diff>

<commit_message>
Fixed template for Shuttle driver expansion
</commit_message>
<xml_diff>
--- a/ScheduleTemplate.xlsx
+++ b/ScheduleTemplate.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brian/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACF09C29-BC5B-F249-9EF0-87FCD773725C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{738E25E4-E8F8-4842-B494-85063A87A65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9940" yWindow="800" windowWidth="24260" windowHeight="21440" xr2:uid="{FD7B0050-CE21-43C8-88B0-92BFB0830FBD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="51">
   <si>
     <t>Holiday Inn Express Vancouver Airport - Schedule</t>
   </si>
@@ -128,15 +128,6 @@
     <t>JOHN</t>
   </si>
   <si>
-    <t>MICHAEL</t>
-  </si>
-  <si>
-    <t>TOSHIYUKI</t>
-  </si>
-  <si>
-    <t>ED</t>
-  </si>
-  <si>
     <t>**AEROMEX</t>
   </si>
   <si>
@@ -197,25 +188,7 @@
     <t>TRISTAN*</t>
   </si>
   <si>
-    <t>MING</t>
-  </si>
-  <si>
-    <t>RAYMOND</t>
-  </si>
-  <si>
-    <t>ROBENSON*</t>
-  </si>
-  <si>
     <t>CARLA</t>
-  </si>
-  <si>
-    <t>SAMUEL</t>
-  </si>
-  <si>
-    <t>JAKRA</t>
-  </si>
-  <si>
-    <t>RONALD</t>
   </si>
 </sst>
 </file>
@@ -552,20 +525,27 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -573,13 +553,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -917,7 +890,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K58"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="5.6640625" customWidth="1"/>
@@ -958,7 +931,7 @@
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E3" s="6">
         <v>46058</v>
@@ -1018,11 +991,11 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
       <c r="D5" s="8" t="s">
         <v>10</v>
       </c>
@@ -1035,9 +1008,9 @@
       <c r="K5" s="9"/>
     </row>
     <row r="6" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="37"/>
-      <c r="B6" s="38"/>
-      <c r="C6" s="37"/>
+      <c r="A6" s="28"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="28"/>
       <c r="D6" s="8" t="s">
         <v>12</v>
       </c>
@@ -1050,9 +1023,9 @@
       <c r="K6" s="10"/>
     </row>
     <row r="7" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="37"/>
-      <c r="B7" s="38"/>
-      <c r="C7" s="37"/>
+      <c r="A7" s="28"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="28"/>
       <c r="D7" s="8" t="s">
         <v>13</v>
       </c>
@@ -1065,9 +1038,9 @@
       <c r="K7" s="10"/>
     </row>
     <row r="8" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="37"/>
-      <c r="B8" s="38"/>
-      <c r="C8" s="37"/>
+      <c r="A8" s="28"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="28"/>
       <c r="D8" s="8" t="s">
         <v>14</v>
       </c>
@@ -1080,9 +1053,9 @@
       <c r="K8" s="10"/>
     </row>
     <row r="9" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="37"/>
-      <c r="B9" s="38"/>
-      <c r="C9" s="37"/>
+      <c r="A9" s="28"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="28"/>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
       <c r="F9" s="10"/>
@@ -1093,9 +1066,9 @@
       <c r="K9" s="10"/>
     </row>
     <row r="10" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="37"/>
-      <c r="B10" s="38"/>
-      <c r="C10" s="37"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="28"/>
       <c r="D10" s="30"/>
       <c r="E10" s="31"/>
       <c r="F10" s="31"/>
@@ -1106,9 +1079,9 @@
       <c r="K10" s="32"/>
     </row>
     <row r="11" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="37"/>
-      <c r="B11" s="38"/>
-      <c r="C11" s="37"/>
+      <c r="A11" s="28"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="28"/>
       <c r="D11" s="8" t="s">
         <v>15</v>
       </c>
@@ -1121,9 +1094,9 @@
       <c r="K11" s="10"/>
     </row>
     <row r="12" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="37"/>
-      <c r="B12" s="38"/>
-      <c r="C12" s="37"/>
+      <c r="A12" s="28"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="28"/>
       <c r="D12" s="8" t="s">
         <v>16</v>
       </c>
@@ -1136,9 +1109,9 @@
       <c r="K12" s="10"/>
     </row>
     <row r="13" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="37"/>
-      <c r="B13" s="38"/>
-      <c r="C13" s="37"/>
+      <c r="A13" s="28"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="28"/>
       <c r="D13" s="8" t="s">
         <v>17</v>
       </c>
@@ -1151,9 +1124,9 @@
       <c r="K13" s="10"/>
     </row>
     <row r="14" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="37"/>
-      <c r="B14" s="38"/>
-      <c r="C14" s="37"/>
+      <c r="A14" s="28"/>
+      <c r="B14" s="29"/>
+      <c r="C14" s="28"/>
       <c r="D14" s="8" t="s">
         <v>18</v>
       </c>
@@ -1166,9 +1139,9 @@
       <c r="K14" s="10"/>
     </row>
     <row r="15" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="37"/>
-      <c r="B15" s="38"/>
-      <c r="C15" s="37"/>
+      <c r="A15" s="28"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="28"/>
       <c r="D15" s="8"/>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
@@ -1179,9 +1152,9 @@
       <c r="K15" s="10"/>
     </row>
     <row r="16" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="37"/>
-      <c r="B16" s="38"/>
-      <c r="C16" s="37"/>
+      <c r="A16" s="28"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="28"/>
       <c r="D16" s="30"/>
       <c r="E16" s="31"/>
       <c r="F16" s="31"/>
@@ -1192,9 +1165,9 @@
       <c r="K16" s="32"/>
     </row>
     <row r="17" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="37"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="37"/>
+      <c r="A17" s="28"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="28"/>
       <c r="D17" s="8" t="s">
         <v>19</v>
       </c>
@@ -1207,11 +1180,11 @@
       <c r="K17" s="9"/>
     </row>
     <row r="18" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="37"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="37"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="28"/>
       <c r="D18" s="8" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="10"/>
@@ -1222,11 +1195,11 @@
       <c r="K18" s="9"/>
     </row>
     <row r="19" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="37"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="37"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="28"/>
       <c r="D19" s="8" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
@@ -1237,9 +1210,9 @@
       <c r="K19" s="10"/>
     </row>
     <row r="20" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="37"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="37"/>
+      <c r="A20" s="28"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="28"/>
       <c r="D20" s="8" t="s">
         <v>21</v>
       </c>
@@ -1252,9 +1225,9 @@
       <c r="K20" s="10"/>
     </row>
     <row r="21" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="37"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="37"/>
+      <c r="A21" s="28"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="28"/>
       <c r="D21" s="8" t="s">
         <v>22</v>
       </c>
@@ -1267,9 +1240,9 @@
       <c r="K21" s="10"/>
     </row>
     <row r="22" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="37"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="37"/>
+      <c r="A22" s="28"/>
+      <c r="B22" s="29"/>
+      <c r="C22" s="28"/>
       <c r="D22" s="8"/>
       <c r="E22" s="10"/>
       <c r="F22" s="9"/>
@@ -1280,9 +1253,9 @@
       <c r="K22" s="10"/>
     </row>
     <row r="23" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="37"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="37"/>
+      <c r="A23" s="28"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="28"/>
       <c r="D23" s="11" t="s">
         <v>23</v>
       </c>
@@ -1295,9 +1268,9 @@
       <c r="K23" s="12"/>
     </row>
     <row r="24" spans="1:11" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="37"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="37"/>
+      <c r="A24" s="28"/>
+      <c r="B24" s="29"/>
+      <c r="C24" s="28"/>
       <c r="D24" s="30"/>
       <c r="E24" s="31"/>
       <c r="F24" s="31"/>
@@ -1308,9 +1281,9 @@
       <c r="K24" s="32"/>
     </row>
     <row r="25" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="37"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="37"/>
+      <c r="A25" s="28"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="28"/>
       <c r="D25" s="8" t="s">
         <v>24</v>
       </c>
@@ -1367,9 +1340,9 @@
       <c r="K27" s="19"/>
     </row>
     <row r="28" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="27"/>
-      <c r="B28" s="28"/>
-      <c r="C28" s="29"/>
+      <c r="A28" s="33"/>
+      <c r="B28" s="34"/>
+      <c r="C28" s="35"/>
       <c r="D28" s="10" t="s">
         <v>27</v>
       </c>
@@ -1382,9 +1355,9 @@
       <c r="K28" s="19"/>
     </row>
     <row r="29" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="27"/>
-      <c r="B29" s="28"/>
-      <c r="C29" s="29"/>
+      <c r="A29" s="33"/>
+      <c r="B29" s="34"/>
+      <c r="C29" s="35"/>
       <c r="D29" s="10" t="s">
         <v>28</v>
       </c>
@@ -1397,9 +1370,9 @@
       <c r="K29" s="19"/>
     </row>
     <row r="30" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="27"/>
-      <c r="B30" s="28"/>
-      <c r="C30" s="29"/>
+      <c r="A30" s="33"/>
+      <c r="B30" s="34"/>
+      <c r="C30" s="35"/>
       <c r="D30" s="10" t="s">
         <v>29</v>
       </c>
@@ -1412,484 +1385,336 @@
       <c r="K30" s="19"/>
     </row>
     <row r="31" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="27"/>
-      <c r="B31" s="28"/>
-      <c r="C31" s="29"/>
-      <c r="D31" s="10" t="s">
+      <c r="A31" s="33"/>
+      <c r="B31" s="34"/>
+      <c r="C31" s="35"/>
+      <c r="D31" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="19"/>
-      <c r="I31" s="19"/>
-      <c r="J31" s="19"/>
-      <c r="K31" s="19"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="13"/>
+      <c r="J31" s="13"/>
+      <c r="K31" s="13"/>
     </row>
     <row r="32" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="27"/>
-      <c r="B32" s="28"/>
-      <c r="C32" s="29"/>
-      <c r="D32" s="10" t="s">
+      <c r="A32" s="23"/>
+      <c r="B32" s="24"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="19"/>
-      <c r="I32" s="19"/>
-      <c r="J32" s="19"/>
-      <c r="K32" s="19"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
     </row>
     <row r="33" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="27"/>
-      <c r="B33" s="28"/>
-      <c r="C33" s="29"/>
-      <c r="D33" s="10" t="s">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="15"/>
+      <c r="I33" s="14"/>
+      <c r="J33" s="14"/>
+      <c r="K33" s="14"/>
+    </row>
+    <row r="34" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="19"/>
-      <c r="J33" s="19"/>
-      <c r="K33" s="19"/>
-    </row>
-    <row r="34" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="27"/>
-      <c r="B34" s="28"/>
-      <c r="C34" s="29"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="22"/>
       <c r="D34" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="E34" s="19"/>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="19"/>
-      <c r="I34" s="19"/>
-      <c r="J34" s="19"/>
-      <c r="K34" s="19"/>
+        <v>33</v>
+      </c>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="16"/>
+      <c r="I34" s="16"/>
+      <c r="J34" s="10"/>
+      <c r="K34" s="10"/>
     </row>
     <row r="35" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="27"/>
-      <c r="B35" s="28"/>
-      <c r="C35" s="29"/>
+      <c r="A35" s="33"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="35"/>
       <c r="D35" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="E35" s="19"/>
-      <c r="F35" s="19"/>
-      <c r="G35" s="19"/>
-      <c r="H35" s="19"/>
-      <c r="I35" s="19"/>
-      <c r="J35" s="19"/>
-      <c r="K35" s="19"/>
+        <v>34</v>
+      </c>
+      <c r="E35" s="10"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="17"/>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
+      <c r="J35" s="17"/>
+      <c r="K35" s="10"/>
     </row>
     <row r="36" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="27"/>
-      <c r="B36" s="28"/>
-      <c r="C36" s="29"/>
+      <c r="A36" s="33"/>
+      <c r="B36" s="34"/>
+      <c r="C36" s="35"/>
       <c r="D36" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="E36" s="19"/>
-      <c r="F36" s="19"/>
-      <c r="G36" s="19"/>
-      <c r="H36" s="19"/>
-      <c r="I36" s="19"/>
-      <c r="J36" s="19"/>
-      <c r="K36" s="19"/>
+        <v>35</v>
+      </c>
+      <c r="E36" s="17"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="17"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="10"/>
+      <c r="J36" s="17"/>
+      <c r="K36" s="17"/>
     </row>
     <row r="37" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="27"/>
-      <c r="B37" s="28"/>
-      <c r="C37" s="29"/>
+      <c r="A37" s="33"/>
+      <c r="B37" s="34"/>
+      <c r="C37" s="35"/>
       <c r="D37" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="E37" s="19"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="19"/>
-      <c r="H37" s="19"/>
-      <c r="I37" s="19"/>
-      <c r="J37" s="19"/>
-      <c r="K37" s="19"/>
+        <v>36</v>
+      </c>
+      <c r="E37" s="10"/>
+      <c r="F37" s="10"/>
+      <c r="G37" s="17"/>
+      <c r="H37" s="17"/>
+      <c r="I37" s="10"/>
+      <c r="J37" s="10"/>
+      <c r="K37" s="10"/>
     </row>
     <row r="38" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="27"/>
-      <c r="B38" s="28"/>
-      <c r="C38" s="29"/>
+      <c r="A38" s="33"/>
+      <c r="B38" s="34"/>
+      <c r="C38" s="35"/>
       <c r="D38" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="E38" s="19"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19"/>
-      <c r="H38" s="19"/>
-      <c r="I38" s="19"/>
-      <c r="J38" s="19"/>
-      <c r="K38" s="19"/>
+        <v>37</v>
+      </c>
+      <c r="E38" s="17"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="10"/>
+      <c r="J38" s="17"/>
+      <c r="K38" s="10"/>
     </row>
     <row r="39" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="27"/>
-      <c r="B39" s="28"/>
-      <c r="C39" s="29"/>
+      <c r="A39" s="33"/>
+      <c r="B39" s="34"/>
+      <c r="C39" s="35"/>
       <c r="D39" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="E39" s="19"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="19"/>
-      <c r="J39" s="19"/>
-      <c r="K39" s="19"/>
+        <v>38</v>
+      </c>
+      <c r="E39" s="17"/>
+      <c r="F39" s="10"/>
+      <c r="G39" s="10"/>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="17"/>
+      <c r="K39" s="10"/>
     </row>
     <row r="40" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="27"/>
-      <c r="B40" s="28"/>
-      <c r="C40" s="29"/>
-      <c r="D40" s="10"/>
-      <c r="E40" s="19"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="19"/>
-      <c r="H40" s="19"/>
-      <c r="I40" s="19"/>
-      <c r="J40" s="19"/>
-      <c r="K40" s="19"/>
+      <c r="A40" s="33"/>
+      <c r="B40" s="34"/>
+      <c r="C40" s="35"/>
+      <c r="D40" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="E40" s="17"/>
+      <c r="F40" s="10"/>
+      <c r="G40" s="10"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="17"/>
+      <c r="K40" s="10"/>
     </row>
     <row r="41" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="27"/>
-      <c r="B41" s="28"/>
-      <c r="C41" s="29"/>
-      <c r="D41" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="E41" s="13"/>
-      <c r="F41" s="13"/>
-      <c r="G41" s="13"/>
-      <c r="H41" s="13"/>
-      <c r="I41" s="13"/>
-      <c r="J41" s="13"/>
-      <c r="K41" s="13"/>
+      <c r="A41" s="23"/>
+      <c r="B41" s="24"/>
+      <c r="C41" s="25"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10"/>
+      <c r="J41" s="10"/>
+      <c r="K41" s="10"/>
     </row>
     <row r="42" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="23"/>
-      <c r="B42" s="24"/>
-      <c r="C42" s="25"/>
-      <c r="D42" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="3"/>
-      <c r="H42" s="3"/>
-      <c r="I42" s="3"/>
-      <c r="J42" s="3"/>
-      <c r="K42" s="3"/>
+      <c r="A42" s="1"/>
+      <c r="B42" s="1"/>
+      <c r="C42" s="1"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5"/>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5"/>
+      <c r="K42" s="5"/>
     </row>
     <row r="43" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="1"/>
-      <c r="B43" s="1"/>
-      <c r="C43" s="1"/>
-      <c r="D43" s="14"/>
-      <c r="E43" s="14"/>
-      <c r="F43" s="14"/>
-      <c r="G43" s="14"/>
-      <c r="H43" s="15"/>
-      <c r="I43" s="14"/>
-      <c r="J43" s="14"/>
-      <c r="K43" s="14"/>
+      <c r="A43" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="B43" s="21"/>
+      <c r="C43" s="22"/>
+      <c r="D43" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E43" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="F43" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="I43" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="J43" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="K43" s="10" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="44" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="B44" s="21"/>
-      <c r="C44" s="22"/>
-      <c r="D44" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
-      <c r="H44" s="16"/>
-      <c r="I44" s="16"/>
-      <c r="J44" s="10"/>
-      <c r="K44" s="10"/>
+      <c r="A44" s="37"/>
+      <c r="B44" s="38"/>
+      <c r="C44" s="35"/>
+      <c r="D44" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E44" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="G44" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="H44" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="I44" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="J44" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="K44" s="10" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="45" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="27"/>
-      <c r="B45" s="28"/>
-      <c r="C45" s="29"/>
-      <c r="D45" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E45" s="10"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="10"/>
-      <c r="I45" s="10"/>
-      <c r="J45" s="17"/>
+      <c r="A45" s="23"/>
+      <c r="B45" s="24"/>
+      <c r="C45" s="25"/>
+      <c r="D45" s="17"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="18"/>
+      <c r="G45" s="18"/>
+      <c r="H45" s="18"/>
+      <c r="I45" s="18"/>
+      <c r="J45" s="18"/>
       <c r="K45" s="10"/>
     </row>
     <row r="46" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="27"/>
-      <c r="B46" s="28"/>
-      <c r="C46" s="29"/>
-      <c r="D46" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="E46" s="17"/>
-      <c r="F46" s="10"/>
-      <c r="G46" s="17"/>
-      <c r="H46" s="17"/>
-      <c r="I46" s="10"/>
-      <c r="J46" s="17"/>
-      <c r="K46" s="17"/>
+      <c r="A46" s="1"/>
+      <c r="B46" s="1"/>
+      <c r="C46" s="1"/>
+      <c r="D46" s="14"/>
+      <c r="E46" s="14"/>
+      <c r="F46" s="14"/>
+      <c r="G46" s="5"/>
+      <c r="H46" s="14"/>
+      <c r="I46" s="14"/>
+      <c r="J46" s="14"/>
+      <c r="K46" s="14"/>
     </row>
     <row r="47" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="27"/>
-      <c r="B47" s="28"/>
-      <c r="C47" s="29"/>
-      <c r="D47" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="E47" s="10"/>
-      <c r="F47" s="10"/>
-      <c r="G47" s="17"/>
-      <c r="H47" s="17"/>
-      <c r="I47" s="10"/>
-      <c r="J47" s="10"/>
-      <c r="K47" s="10"/>
+      <c r="A47" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="B47" s="21"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E47" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="F47" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="G47" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="H47" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="I47" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="J47" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="K47" s="10" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="48" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="27"/>
-      <c r="B48" s="28"/>
-      <c r="C48" s="29"/>
-      <c r="D48" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E48" s="17"/>
-      <c r="F48" s="10"/>
-      <c r="G48" s="10"/>
-      <c r="H48" s="10"/>
-      <c r="I48" s="10"/>
-      <c r="J48" s="17"/>
-      <c r="K48" s="10"/>
-    </row>
-    <row r="49" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="27"/>
-      <c r="B49" s="28"/>
-      <c r="C49" s="29"/>
-      <c r="D49" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="E49" s="17"/>
-      <c r="F49" s="10"/>
-      <c r="G49" s="10"/>
-      <c r="H49" s="10"/>
-      <c r="I49" s="10"/>
-      <c r="J49" s="17"/>
-      <c r="K49" s="10"/>
-    </row>
-    <row r="50" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="27"/>
-      <c r="B50" s="28"/>
-      <c r="C50" s="29"/>
-      <c r="D50" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="E50" s="17"/>
-      <c r="F50" s="10"/>
-      <c r="G50" s="10"/>
-      <c r="H50" s="10"/>
-      <c r="I50" s="10"/>
-      <c r="J50" s="17"/>
-      <c r="K50" s="10"/>
-    </row>
-    <row r="51" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="23"/>
-      <c r="B51" s="24"/>
-      <c r="C51" s="25"/>
-      <c r="D51" s="10"/>
-      <c r="E51" s="10"/>
-      <c r="F51" s="10"/>
-      <c r="G51" s="10"/>
-      <c r="H51" s="10"/>
-      <c r="I51" s="10"/>
-      <c r="J51" s="10"/>
-      <c r="K51" s="10"/>
-    </row>
-    <row r="52" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="1"/>
-      <c r="B52" s="1"/>
-      <c r="C52" s="1"/>
-      <c r="D52" s="5"/>
-      <c r="E52" s="5"/>
-      <c r="F52" s="5"/>
-      <c r="G52" s="5"/>
-      <c r="H52" s="5"/>
-      <c r="I52" s="5"/>
-      <c r="J52" s="5"/>
-      <c r="K52" s="5"/>
-    </row>
-    <row r="53" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="33" t="s">
-        <v>42</v>
-      </c>
-      <c r="B53" s="21"/>
-      <c r="C53" s="22"/>
-      <c r="D53" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="E53" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="F53" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="G53" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="H53" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="I53" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="J53" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="K53" s="10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="34"/>
-      <c r="B54" s="35"/>
-      <c r="C54" s="29"/>
-      <c r="D54" s="17" t="s">
+      <c r="A48" s="23"/>
+      <c r="B48" s="24"/>
+      <c r="C48" s="25"/>
+      <c r="D48" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="E54" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="F54" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="G54" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="H54" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="I54" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="J54" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="K54" s="10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="23"/>
-      <c r="B55" s="24"/>
-      <c r="C55" s="25"/>
-      <c r="D55" s="17"/>
-      <c r="E55" s="18"/>
-      <c r="F55" s="18"/>
-      <c r="G55" s="18"/>
-      <c r="H55" s="18"/>
-      <c r="I55" s="18"/>
-      <c r="J55" s="18"/>
-      <c r="K55" s="10"/>
-    </row>
-    <row r="56" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="1"/>
-      <c r="B56" s="1"/>
-      <c r="C56" s="1"/>
-      <c r="D56" s="14"/>
-      <c r="E56" s="14"/>
-      <c r="F56" s="14"/>
-      <c r="G56" s="5"/>
-      <c r="H56" s="14"/>
-      <c r="I56" s="14"/>
-      <c r="J56" s="14"/>
-      <c r="K56" s="14"/>
-    </row>
-    <row r="57" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="20" t="s">
+      <c r="E48" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="B57" s="21"/>
-      <c r="C57" s="22"/>
-      <c r="D57" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="E57" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="F57" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="G57" s="10" t="s">
+      <c r="F48" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="H57" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="I57" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="J57" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="K57" s="10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="23"/>
-      <c r="B58" s="24"/>
-      <c r="C58" s="25"/>
-      <c r="D58" s="17" t="s">
-        <v>48</v>
-      </c>
-      <c r="E58" s="10" t="s">
-        <v>49</v>
-      </c>
-      <c r="F58" s="10" t="s">
+      <c r="G48" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="G58" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="H58" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="I58" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="J58" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="K58" s="9" t="s">
-        <v>49</v>
+      <c r="H48" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="I48" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="J48" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="K48" s="9" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A57:C58"/>
+    <mergeCell ref="A47:C48"/>
     <mergeCell ref="D1:K2"/>
     <mergeCell ref="A5:C25"/>
     <mergeCell ref="D24:K24"/>
-    <mergeCell ref="A27:C42"/>
-    <mergeCell ref="A44:C51"/>
-    <mergeCell ref="A53:C55"/>
+    <mergeCell ref="A27:C32"/>
+    <mergeCell ref="A34:C41"/>
+    <mergeCell ref="A43:C45"/>
     <mergeCell ref="D10:K10"/>
     <mergeCell ref="D16:K16"/>
   </mergeCells>

</xml_diff>

<commit_message>
updated dev database and support for 24h time support
</commit_message>
<xml_diff>
--- a/ScheduleTemplate.xlsx
+++ b/ScheduleTemplate.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brian/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{738E25E4-E8F8-4842-B494-85063A87A65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7010D8FC-10FB-B440-BE72-F0A392A75D90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9940" yWindow="800" windowWidth="24260" windowHeight="21440" xr2:uid="{FD7B0050-CE21-43C8-88B0-92BFB0830FBD}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="49">
   <si>
     <t>Holiday Inn Express Vancouver Airport - Schedule</t>
   </si>
@@ -152,9 +152,6 @@
     <t>MERVE*</t>
   </si>
   <si>
-    <t>AYAKO</t>
-  </si>
-  <si>
     <t>Maintenance</t>
   </si>
   <si>
@@ -186,9 +183,6 @@
   </si>
   <si>
     <t>TRISTAN*</t>
-  </si>
-  <si>
-    <t>CARLA</t>
   </si>
 </sst>
 </file>
@@ -931,7 +925,7 @@
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E3" s="6">
         <v>46058</v>
@@ -1184,7 +1178,7 @@
       <c r="B18" s="29"/>
       <c r="C18" s="28"/>
       <c r="D18" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="10"/>
@@ -1199,7 +1193,7 @@
       <c r="B19" s="29"/>
       <c r="C19" s="28"/>
       <c r="D19" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
@@ -1508,9 +1502,7 @@
       <c r="A39" s="33"/>
       <c r="B39" s="34"/>
       <c r="C39" s="35"/>
-      <c r="D39" s="10" t="s">
-        <v>38</v>
-      </c>
+      <c r="D39" s="10"/>
       <c r="E39" s="17"/>
       <c r="F39" s="10"/>
       <c r="G39" s="10"/>
@@ -1523,9 +1515,7 @@
       <c r="A40" s="33"/>
       <c r="B40" s="34"/>
       <c r="C40" s="35"/>
-      <c r="D40" s="10" t="s">
-        <v>50</v>
-      </c>
+      <c r="D40" s="10"/>
       <c r="E40" s="17"/>
       <c r="F40" s="10"/>
       <c r="G40" s="10"/>
@@ -1562,15 +1552,15 @@
     </row>
     <row r="43" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B43" s="21"/>
       <c r="C43" s="22"/>
       <c r="D43" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="E43" s="10" t="s">
         <v>40</v>
-      </c>
-      <c r="E43" s="10" t="s">
-        <v>41</v>
       </c>
       <c r="F43" s="18" t="s">
         <v>11</v>
@@ -1579,16 +1569,16 @@
         <v>11</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I43" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J43" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K43" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -1596,7 +1586,7 @@
       <c r="B44" s="38"/>
       <c r="C44" s="35"/>
       <c r="D44" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E44" s="18" t="s">
         <v>11</v>
@@ -1648,33 +1638,33 @@
     </row>
     <row r="47" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B47" s="21"/>
       <c r="C47" s="22"/>
       <c r="D47" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F47" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G47" s="10" t="s">
         <v>20</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="I47" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J47" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K47" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -1682,10 +1672,10 @@
       <c r="B48" s="24"/>
       <c r="C48" s="25"/>
       <c r="D48" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="E48" s="10" t="s">
         <v>45</v>
-      </c>
-      <c r="E48" s="10" t="s">
-        <v>46</v>
       </c>
       <c r="F48" s="10" t="s">
         <v>20</v>
@@ -1694,16 +1684,16 @@
         <v>20</v>
       </c>
       <c r="H48" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I48" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J48" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="K48" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>